<commit_message>
A kérdések átírt szövege a szerkesztett Excelből
Nyelvi átdolgozás mindhárom pályán (új jelenetcímek, helyzetleírások,
válaszok, kiértékelések), két pontmódosítással (politikai 7B, 8C).
Javítva: politikai 7 (a „tizenkét település" kimaradt, ellentmondott a B
válasz „harmadával" állításának), vállalati 6 (kétértelmű pénzmondat),
katonai 7 („folyó feletti tározás").

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/szerkesztes/kerdesek.xlsx
+++ b/szerkesztes/kerdesek.xlsx
@@ -778,7 +778,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Kérsz két hetet, mielőtt bármiről szavaznátok. Ez alatt leírjátok, mit akartok pontosan elérni — spórolást, jobb iskolákat vagy mindkettőt —, és mit semmiképp nem szeretnétek feláldozni.</t>
+          <t>Két hetet kérsz, mielőtt bármiről szavaznátok. Ezalatt leírjátok, pontosan mit akartok elérni — megtakarítást, jobb iskolákat vagy mindkettőt —, és mi az, amit semmiképp sem akartok feláldozni.</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Ez a PrOACT-modell első két lépése: a probléma pontos megfogalmazása és a célok teljes listájának összeírása, mielőtt bármilyen megoldást mérlegelnénk. A táblázat a megoldást már készen hozta, te viszont visszaléptél a kérdéshez: mit akarunk valójában? Ennek ára a két hét csúszás és egy türelmetlen frakcióvezető.</t>
+          <t>Ez a PrOACT-modell első két lépése: pontosan megfogalmazni a problémát, és összeírni az összes célt, mielőtt bármilyen megoldást mérlegelnénk. A táblázat kész megoldással érkezett, te viszont visszaléptél a kérdéshez: mit akarunk valójában? Ennek ára két hét csúszás és egy türelmetlen frakcióvezető.</t>
         </is>
       </c>
     </row>
@@ -870,7 +870,7 @@
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>Egy parlamenti bizottság elnöke vagy. A kormány takarékossági csomagja negyven kis falusi iskola bezárását javasolja: a gyerekeket busszal vinnék a közeli városokba. Tíz hét alatt kell végigvinned a javaslatot a bizottságon és a parlamenten, miközben a falvak, a pedagógusok, a pártod és a sajtó is figyel.</t>
+          <t>Egy parlamenti bizottság elnöke vagy. A kormány takarékossági csomagja negyven kis falusi iskola bezárását javasolja: a gyerekeket busszal vinnék be a közeli városokba. Tíz héted van arra, hogy a javaslatot végigvidd a bizottságon és a parlamenten, miközben a falvak, a pedagógusok, a pártod és a sajtó is minden lépésedet figyeli.</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>A Meridian Kft. ügyfélszolgálati igazgatója vagy. A cég legnagyobb ügyfele, egy országos patikalánc, három hónapot adott: ha addig nem javul a kiszolgálás, felmondja a szerződést, amely a bevétel negyedét hozza. A csapatod fáradt, az osztályok egymást hibáztatják, a vezérigazgató pedig eredményt vár.</t>
+          <t>A Meridian Kft. ügyfélszolgálati igazgatója vagy. A cég legnagyobb ügyfele, egy országos patikalánc, három hónapot adott: ha addig nem javul a kiszolgálás, felmondja a szerződést, amelyből a cég bevételének negyede származik. A csapatod kimerült, az osztályok egymást hibáztatják, a vezérigazgató pedig eredményeket vár.</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>A 3. műszaki ezred parancsnoka vagy. Rekordmagas árhullám közeledik a Tiszán, és az ezredet egy háromezres folyóparti város, Tiszaszög és a környező tanyák védelmére vezénylik. Tizenkét nap áll rendelkezésre: az állomány fáradt, a gépek kevesek, a helyiek félnek, és minden döntésed emberek otthonáról szól.</t>
+          <t>A 3. műszaki ezred parancsnoka vagy. Rekordmagas árhullám közeleg a Tiszán, és az ezredet egy háromezer lakosú folyóparti város, Tiszaszög és a környező tanyák védelmére vezénylik. Tizenkét napotok van: az állomány fáradt, kevés a gép, a helyiek félnek, és minden döntésed emberek otthonáról szól.</t>
         </is>
       </c>
     </row>
@@ -1016,12 +1016,12 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>A táblázat</t>
+          <t>A minisztérium táblázata</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Hétfő reggel megérkezik a minisztérium anyaga: egyetlen táblázat. Negyven iskola neve, a tanulók száma, és mellette, mennyit spórol az állam, ha bezárják őket. A bizottság három tagja már az első percben összevész rajta, a pártod frakcióvezetője pedig üzen: jó lenne egy hónap alatt letudni. Mielőtt bárki szavazna, neked kell eldöntened, hogyan kezditek.</t>
+          <t>Hétfő reggel megérkezik a minisztérium anyaga: egyetlen táblázat. Benne a negyven iskola neve, a tanulók száma, és hogy mennyit spórol az állam, ha bezárják őket. A bizottság három tagja már az első percekben összevitatkozik rajta, a frakcióvezetőd pedig üzeni, hogy jó lenne egy hónap alatt lezárni az ügyet. Mielőtt bárki szavazna, neked kell eldöntened, hogyan fogjatok hozzá.</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>Még aznap nyilatkozol: amíg te vagy a bizottság elnöke, egyetlen falu sem veszíti el az iskoláját. A falvak hálásak, a sajtó felkapja, és a tárgyalásokon erős pozícióból indulsz.</t>
+          <t>Még aznap nyilatkozatot teszel: amíg te vezeted a bizottságot, egyetlen falu sem veszíti el az iskoláját. A falvak hálásak, a sajtó felkapja a hírt, és erős pozícióból ülsz le tárgyalni.</t>
         </is>
       </c>
       <c r="F2" s="11" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Snowden és Boone szerint egyszerű helyzetben létezik egy helyes válasz, amelyet elég kimondani; komplex helyzetben viszont nincs ilyen, az okok és a következmények csak menet közben rajzolódnak ki. Az ígérettel egyszerűnek kezelted az ügyet. Most erős vagy, de ha a számok később mást mutatnak, a saját szavad lesz a legnagyobb ellenfeled.</t>
+          <t>Snowden és Boone szerint egyszerű helyzetben létezik egyetlen helyes válasz, amelyet elég kimondani. Komplex helyzetben viszont nincs ilyen: az okok és a következmények csak menet közben rajzolódnak ki. Az ígéreteddel úgy kezelted az ügyet, mintha egyszerű volna. Most erős a pozíciód, de ha a számok később mást mutatnak, a saját szavad fordul ellened.</t>
         </is>
       </c>
       <c r="H2" s="12" t="n">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="E3" s="17" t="inlineStr">
         <is>
-          <t>A táblázatot fogadod el kiindulópontnak, és a bizottság csak azt vitatja meg, melyik iskola kerüljön le a listáról. Így gyorsan haladtok, és a pártod is elégedett.</t>
+          <t>Elfogadod kiindulópontnak a táblázatot, és a bizottság csak arról vitázik, melyik iskola kerüljön le a listáról. Így gyorsan haladtok, és a pártod is elégedett.</t>
         </is>
       </c>
       <c r="F3" s="17" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
-          <t>Simon megkülönböztetése szerint a jól strukturált döntésnél csak az a kérdés, hogyan oldjuk meg, a rosszul strukturáltnál viszont még az sem világos, mi a probléma. Az iskolabezárás tipikusan rosszul strukturált: nem egyértelmű, hogy költség-, oktatási vagy közösségi kérdés. Ha jól strukturáltként kezeled, gyors leszel, de a valódi vitát csak elhalasztod.</t>
+          <t>Simon megkülönböztetése szerint egy jól strukturált döntésnél csak az a kérdés, hogyan oldjuk meg a problémát; a rosszul strukturáltnál még az sem világos, mi maga a probléma. Az iskolabezárás tipikusan ilyen: nem egyértelmű, hogy költségvetési, oktatási vagy közösségi kérdésről van-e szó. Ha jól strukturáltként kezeled, gyorsan haladsz, de a valódi vitát csak elodázod.</t>
         </is>
       </c>
       <c r="H3" s="18" t="n">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="E4" s="17" t="inlineStr">
         <is>
-          <t>Kérsz két hetet, mielőtt bármiről szavaznátok. Ez alatt leírjátok, mit akartok pontosan elérni — spórolást, jobb iskolákat vagy mindkettőt —, és mit semmiképp nem szeretnétek feláldozni.</t>
+          <t>Két hetet kérsz, mielőtt bármiről szavaznátok. Ezalatt leírjátok, pontosan mit akartok elérni — megtakarítást, jobb iskolákat vagy mindkettőt —, és mi az, amit semmiképp sem akartok feláldozni.</t>
         </is>
       </c>
       <c r="F4" s="17" t="inlineStr">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="G4" s="17" t="inlineStr">
         <is>
-          <t>Ez a PrOACT-modell első két lépése: a probléma pontos megfogalmazása és a célok teljes listájának összeírása, mielőtt bármilyen megoldást mérlegelnénk. A táblázat a megoldást már készen hozta, te viszont visszaléptél a kérdéshez: mit akarunk valójában? Ennek ára a két hét csúszás és egy türelmetlen frakcióvezető.</t>
+          <t>Ez a PrOACT-modell első két lépése: pontosan megfogalmazni a problémát, és összeírni az összes célt, mielőtt bármilyen megoldást mérlegelnénk. A táblázat kész megoldással érkezett, te viszont visszaléptél a kérdéshez: mit akarunk valójában? Ennek ára két hét csúszás és egy türelmetlen frakcióvezető.</t>
         </is>
       </c>
       <c r="H4" s="18" t="n">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="E5" s="17" t="inlineStr">
         <is>
-          <t>Mielőtt bármit mondanál a bizottságban, egy hét alatt végiglátogatsz öt érintett falut, hogy a saját szemeddel lásd, miről szól a táblázat.</t>
+          <t>Mielőtt bármit mondanál a bizottságban, egy hét alatt végiglátogatsz öt érintett falut, hogy a saját szemeddel lásd, mi áll a táblázat számai mögött.</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg tíz vezetői szerepe közül ez az információgyűjtő: a vezető maga megy el oda, ahol első kézből tudhat meg valamit. A terepen olyat látsz, amit a táblázat nem mutat. Az ára, hogy közben a bizottság nélküled kezd vitatkozni, és a tagjaid kimaradnak abból, amit te megtapasztalsz.</t>
+          <t>Mintzberg tíz vezetői szerepe közül ez az információgyűjtő szerep: a vezető maga megy oda, ahol első kézből tájékozódhat. A terepen olyasmit is látsz, amit a táblázat nem mutat meg. Az ára, hogy a bizottság közben nélküled kezd vitatkozni, és a tagok semmit sem látnak abból, amit te tapasztalsz.</t>
         </is>
       </c>
       <c r="H5" s="18" t="n">
@@ -1218,12 +1218,12 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>A falugyűlés</t>
+          <t>Falugyűlés Bükkfalván</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>A táblázat kiszivárgott. Szombaton Bükkfalván, a listán szereplő egyik faluban háromszáz ember gyűlik össze a kultúrházban, és téged is meghívnak. A szervező előre szól: a szülők dühösek, és arra akarnak választ, megmarad-e az iskolájuk. A kamerák is ott lesznek.</t>
+          <t>A táblázat kiszivárgott. Szombaton Bükkfalván, az egyik listán szereplő faluban háromszáz ember gyűlik össze a kultúrházban, és téged is meghívnak. A szervező előre figyelmeztet: a szülők dühösek, és arra várnak választ, hogy megmarad-e az iskolájuk. A sajtó is ott lesz.</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Elmész, és megígéred, hogy Bükkfalva iskolája marad. A terem tapsol, a hír estére mindenhol ott van.</t>
+          <t>Elmész, és megígéred, hogy Bükkfalva iskolája megmarad. A terem tapsol, estére pedig már mindenhol erről szól a hír.</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>A diszkontálás az a hajlamunk, hogy a közeli, most jelen lévő dolgokat felértékeljük, a távolabbiakat pedig leértékeljük. A dühös terem itt és most van, a harminckilenc másik falu és a költségvetés viszont távolinak tűnik. Az ígéret ma békét hoz, holnap viszont mindenki ugyanezt fogja kérni tőled.</t>
+          <t>A diszkontálás az a hajlamunk, hogy ami közel van és most történik, azt túlértékeljük, ami távolabb esik, azt pedig alábecsüljük. A dühös terem itt és most van előtted, a többi harminckilenc falu és a költségvetés viszont messzinek tűnik. Az ígéret ma békét hoz, holnap viszont mindenki ugyanezt fogja kérni tőled.</t>
         </is>
       </c>
       <c r="H6" s="12" t="n">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="E7" s="17" t="inlineStr">
         <is>
-          <t>Elmész, és felajánlod, hogy a falu két hónap alatt dolgozzon ki saját javaslatot, amit a bizottság ugyanúgy megvizsgál, mint a minisztériumét. Ez lassítja a menetrendet, és a pártod nem fog örülni.</t>
+          <t>Elmész, és felajánlod, hogy a falu két hónap alatt dolgozzon ki saját javaslatot, amelyet a bizottság ugyanolyan komolyan megvizsgál, mint a minisztériumét. Ez lelassítja a menetrendet, és a pártod sem fog örülni neki.</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>A részvételi létra azt mutatja, mennyire valódi az érintettek bevonása: a puszta tájékoztatástól egészen addig, amikor a döntés egy részét ténylegesen rájuk bízzuk. Te a létra felső fokára léptél, a falu nemcsak véleményt mondhat, hanem saját javaslattal is beszállhat. Az ár a két hónap csúszás és egy frakció, amely úgy érzi, kiengedted a kezedből az ügyet.</t>
+          <t>A részvételi létra azt mutatja meg, mennyire valódi az érintettek bevonása: a puszta tájékoztatástól egészen addig, amikor a döntés egy részét ténylegesen rájuk bízzuk. Te a létra felső fokára léptél: a falu nemcsak véleményt mondhat, hanem saját javaslatot is tehet. Az ár két hónap csúszás és egy frakció, amely úgy érzi, kiengedted a kezedből az ügyet.</t>
         </is>
       </c>
       <c r="H7" s="18" t="n">
@@ -1318,7 +1318,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="76" customHeight="1">
+    <row r="8" ht="90" customHeight="1">
       <c r="A8" s="15" t="n"/>
       <c r="B8" s="16" t="n"/>
       <c r="C8" s="17" t="n"/>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="E8" s="17" t="inlineStr">
         <is>
-          <t>Nem mész el személyesen: a minisztérium egyik szakértőjét küldöd, aki számokkal elmagyarázza, miért szükséges az átszervezés. Így nem te leszel a dühös emberek célpontja, és a számokat is pontosabban mondja el.</t>
+          <t>Nem mész el személyesen, hanem a minisztérium egyik szakértőjét küldöd, aki a számokkal elmagyarázza, miért van szükség az átszervezésre. Így nem rád zúdul az emberek dühe, és a számokat is pontosabban ismerteti.</t>
         </is>
       </c>
       <c r="F8" s="17" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg szerint a vezetőnek képviselő szerepe is van: a jelenléte önmagában üzenet, hiszen a tisztsége szimbolikus súlyú. A szakértő pontosabban beszél a számokról, a teremben mégis az marad meg, hogy te nem jöttél el. A távolmaradás megóv egy kellemetlen estétől, és elveszi az esélyt, hogy személyesen építs bizalmat.</t>
+          <t>Mintzberg szerint a vezetőnek képviselő szerepe is van: már a jelenléte is üzenet, mert a tisztségének szimbolikus súlya van. A szakértő pontosabban beszél a számokról, a teremben mégis az marad meg, hogy te nem jöttél el. A távolmaradással megúszol egy kellemetlen estét, de elszalasztod az esélyt, hogy személyesen építs bizalmat.</t>
         </is>
       </c>
       <c r="H8" s="18" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="E9" s="17" t="inlineStr">
         <is>
-          <t>Elmész, végighallgatod őket, és elmondod, hogy még semmi sincs eldöntve — de ígéretet nem teszel. Tudod, hogy ezzel valószínűleg senki nem lesz elégedett.</t>
+          <t>Elmész, végighallgatod őket, és elmondod, hogy még semmi sincs eldöntve — de ígéretet nem teszel. Tudod, hogy ezzel valószínűleg senkit sem fogsz elégedetté tenni.</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg kapcsolattartó szerepében a vezető kapcsolatokat épít a szervezeten kívüliekkel, és közben információt is gyűjt. Ha meghallgatod őket, de nem ígérsz, megőrzöd a mozgásteredet és a hitelességedet. A teremből viszont sokan úgy mennek haza, hogy kiálltál eléjük, és nem mondtál semmit.</t>
+          <t>Mintzberg kapcsolattartó szerepében a vezető a szervezeten kívüliekkel épít kapcsolatot, és közben információt is gyűjt. Ha meghallgatod őket, de nem ígérsz semmit, megőrzöd a mozgásteredet és a hitelességedet. Sokan viszont azzal mennek haza, hogy kiálltál eléjük, de nem mondtál semmit.</t>
         </is>
       </c>
       <c r="H9" s="18" t="n">
@@ -1420,12 +1420,12 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Az ajánlat</t>
+          <t>A buszos cég ajánlata</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>A parlament folyosóján megszólít egy ismert buszos cég vezetője. A cég országszerte pontos, megbízható járatairól híres. Az ajánlata: öt évig ingyen szállítják a gyerekeket a bezárt falvakból, ha a bizottság úgy írja meg a törvényt, hogy a szállítást pályázat nélkül ők kaphassák meg. A szülők legnagyobb félelme éppen az utazás.</t>
+          <t>A parlament folyosóján megszólít egy ismert buszos cég vezetője. A cég országszerte pontos, megbízható járatairól ismert. Az ajánlata: öt évig ingyen szállítják a gyerekeket azokból a falvakból, ahol bezár az iskola, ha a bizottság úgy fogalmazza meg a törvényt, hogy a szállítást pályázat nélkül ők kaphassák meg. A szülők pedig éppen az utazástól félnek a legjobban.</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Megköszönöd, de közlöd, hogy a szállításra nyílt pályázat lesz, akkor is, ha drágább és lassabb. Tudod, hogy így a buszok hónapokkal később indulnak, és addig a szülők aggodalma is megmarad.</t>
+          <t>Megköszönöd az ajánlatot, de jelzed, hogy a szállításra nyílt pályázatot írtok ki, még ha az drágább és lassabb is. Tudod, hogy így a buszok csak hónapokkal később indulnak, és addig a szülők aggodalma sem múlik el.</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>A napfény teszt egyetlen kérdés: jól érezném magam, ha ez a döntés minden részletével együtt holnap nyilvánosságra kerülne? Egy pályázat nélküli, ingyenesnek látszó üzlet nehezen állná ki ezt a próbát. A nyílt pályázat tisztább, de a gyerekek addig bizonytalanságban maradnak, és a megtakarítás is kisebb.</t>
+          <t>A napfény teszt egyetlen kérdés: jól érezném-e magam, ha ez a döntés minden részletével együtt holnap nyilvánosságra kerülne? Egy pályázat nélküli, ingyenesnek látszó üzlet nehezen állná ki ezt a próbát. A nyílt pályázat tisztább megoldás, de a gyerekek addig bizonytalanságban maradnak, és a megtakarítás is kisebb lesz.</t>
         </is>
       </c>
       <c r="H10" s="12" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="E11" s="17" t="inlineStr">
         <is>
-          <t>Elfogadod: a gyerekek biztonságos, ingyenes buszt kapnak, az állam spórol, a szülők megnyugszanak. Úgy gondolod, egy ilyen jó ügyért belefér, hogy most kivételesen nem lesz pályázat.</t>
+          <t>Elfogadod: a gyerekek biztonságos, ingyenes buszt kapnak, az állam spórol, a szülők megnyugszanak. Úgy gondolod, egy ilyen jó ügy érdekében belefér, hogy ezúttal kivételesen ne legyen pályázat.</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet gátló racionalizálásnak nevezi azokat az érveket, amelyekkel egy kétes döntést magunk előtt elfogadhatóvá teszünk. A „jó célt szolgál” az egyik leggyakoribb: az eredmény valóban értékes, de a hozzá vezető út — egy cégnek tett szívesség pályázat nélkül — etikai csapdát rejt. Rövid távon mindenki jól jár, amíg ki nem derül, mi volt az ára.</t>
+          <t>A jegyzet gátló racionalizálásnak nevezi azokat az érveket, amelyekkel egy kétes döntést a saját szemünkben elfogadhatóvá teszünk. A „jó célt szolgál” az egyik leggyakoribb ilyen érv: az eredmény valóban értékes, de az odavezető út — egy cégnek tett, pályázat nélküli szívesség — etikai csapdát rejt. Rövid távon mindenki jól jár, egészen addig, amíg ki nem derül, mi volt az ára.</t>
         </is>
       </c>
       <c r="H11" s="18" t="n">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="E12" s="17" t="inlineStr">
         <is>
-          <t>Nem döntesz egyedül: a következő bizottsági ülésen nyilvánosan ismerteted az ajánlatot, és közösen döntötök róla. Lehet, hogy a cég ezután visszalép, mert nem szereti a nyilvánosságot.</t>
+          <t>Nem döntesz egyedül: a következő bizottsági ülésen nyilvánosan ismerteted az ajánlatot, és közösen döntötök róla. Elképzelhető, hogy a cég ezután visszalép, mert nem kedveli a nyilvánosságot.</t>
         </is>
       </c>
       <c r="F12" s="17" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg információelosztó szerepében a vezető továbbadja a hozzá befutó információt azoknak, akiknek szükségük van rá. Ezzel az ajánlat a bizottság közös ügye lett, nem egy folyosói beszélgetésé. A nyitottság ára, hogy egy jó ajánlat is elveszhet, és a döntés felelősségét megosztod másokkal.</t>
+          <t>Mintzberg információelosztó szerepében a vezető továbbadja a hozzá befutó információt azoknak, akiknek szükségük van rá. Így az ajánlat a bizottság közös ügye lett, nem egy folyosói beszélgetés titka. A nyitottság ára, hogy egy jó ajánlat is elveszhet, és a döntés felelősségén másokkal osztozol.</t>
         </is>
       </c>
       <c r="H12" s="18" t="n">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="E13" s="17" t="inlineStr">
         <is>
-          <t>Egy ennyire megbízható cég ajánlatában nem látsz nagy kockázatot. Négyszemközt azt kéred, tegyenek még jobb ajánlatot, és addig nem szólsz róla senkinek.</t>
+          <t>Egy ennyire megbízható cég ajánlatában nem látsz nagy kockázatot. Négyszemközt arra kéred őket, hogy tegyenek még jobb ajánlatot, és addig senkinek sem szólsz róla.</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>A halo-effektus azt jelenti, hogy egyetlen kiemelkedő tulajdonság alapján alkotunk általános véleményt valakiről. A cég pontos buszjáratai miatt az ajánlatát is megbízhatónak láttad, pedig a kettő nem ugyanaz: a járatok minősége semmit sem mond arról, tisztességes-e egy pályázat nélküli üzlet. A titkos alku jobb feltételeket hozhat, de ha kiderül, az egész bizottságot magával rántja.</t>
+          <t>A halo-effektus azt jelenti, hogy egyetlen kiemelkedő tulajdonság alapján alkotunk általános véleményt valakiről. A cég pontos járatai miatt az ajánlatát is megbízhatónak láttad, pedig a kettőnek nincs köze egymáshoz: a buszok pontossága semmit sem mond arról, tisztességes-e egy pályázat nélküli üzlet. A titkos alku jobb feltételeket hozhat, de ha kiderül, az egész bizottságot magával rántja.</t>
         </is>
       </c>
       <c r="H13" s="18" t="n">
@@ -1622,12 +1622,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>A személyes támadás</t>
+          <t>Személyeskedő támadás a bizottságban</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>A bizottsági vitán felszólal Kardos Ilona, az ellenzék képviselője, aki húsz évig tanított egy falusi iskolában. Hangosan és személyeskedve támad: szerinte azért akarsz iskolákat bezárni, mert soha nem éltél vidéken. A pártodbeli helyetted odasúgja: ne foglalkozz vele, csak a kameráknak játszik. Az egész terem rád néz.</t>
+          <t>A bizottsági vitában felszólal Kardos Ilona, az ellenzék képviselője, aki húsz évig tanított egy falusi iskolában. Hangosan, személyeskedve támad: szerinte csak azért akarsz iskolákat bezárni, mert sosem éltél vidéken. A helyetted, aki egyben a párttársad is, odasúgja, hogy ne foglalkozz vele, csak a kameráknak játszik. Az egész terem rád figyel.</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Szünetet rendelsz el, és négyszemközt próbálsz megegyezni Kardos Ilonával: ha az ő két iskolájának ügyét külön megvizsgáljátok, a nyilvános vitában visszafogja magát.</t>
+          <t>Szünetet rendelsz el, és négyszemközt próbálsz megegyezni Kardos Ilonával: ha az ő két iskolája ügyét külön megvizsgáljátok, ő cserébe visszafogottabb lesz a nyilvános vitában.</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Mintzberg tárgyaló szerepében a vezető egyezkedéssel szerez támogatást vagy nyugalmat. A négyszemközti megállapodás lecsillapíthatja a vitát, és a két iskola ügye is előrébb juthat. A nyilvánosság viszont kimarad belőle: a bizottság többi tagja és a sajtó csak annyit lát, hogy a vita hirtelen elcsendesedett.</t>
+          <t>Mintzberg tárgyaló szerepében a vezető alkuval szerez támogatást vagy nyugalmat. A négyszemközti megállapodás lecsillapíthatja a vitát, és a két iskola ügye is előrébb juthat. A nyilvánosság viszont kimarad belőle: a bizottság többi tagja és a sajtó csak annyit lát, hogy a vita hirtelen elcsendesedett.</t>
         </is>
       </c>
       <c r="H14" s="12" t="n">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>Az alapvető attribúciós hiba az a hajlamunk, hogy mások viselkedését a jellemükkel vagy a szándékukkal magyarázzuk, a helyzet hatását pedig alábecsüljük. Ha Kardos Ilona felszólalását puszta politikai játéknak látod, kimarad, hogy húsz évnyi falusi tapasztalatból beszél. A vita rendezett marad, a mögötte álló valódi aggály viszont válasz nélkül.</t>
+          <t>Az alapvető attribúciós hiba az a hajlamunk, hogy mások viselkedését a jellemükkel vagy a szándékaikkal magyarázzuk, a körülmények hatását pedig alábecsüljük. Ha Kardos Ilona felszólalását puszta politikai színjátéknak látod, elsikkad, hogy húsz év falusi tapasztalatából beszél. A vita rendezett marad, a mögötte meghúzódó valódi aggodalom viszont válasz nélkül.</t>
         </is>
       </c>
       <c r="H15" s="18" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="E16" s="17" t="inlineStr">
         <is>
-          <t>Nyugodtan megkéred, nevezzen meg két iskolát, ahol szerinte hibásak a számok, és felajánlod, hogy azokat jövő héten közösen újraszámoljátok. Ezzel teret adsz neki, és a vita is elhúzódik.</t>
+          <t>Nyugodtan megkéred, hogy nevezzen meg két iskolát, ahol szerinte hibásak a számok, és felajánlod, hogy jövő héten közösen újraszámoljátok őket. Ezzel teret adsz neki, a vita viszont elhúzódik.</t>
         </is>
       </c>
       <c r="F16" s="17" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet kétféle vitamagatartást állít szembe: a pártfogó a saját álláspontját védi és a másikét próbálja elhallgattatni, a vizsgálódó pedig közösen teszteli az érveket. Te az utóbbit választottad: a támadás mögötti tapasztalatot vizsgálható kérdéssé alakítottad. A vita tartalmasabb lesz, de időt visz el, és a párttársaid gyengeségnek láthatják.</t>
+          <t>A jegyzet kétféle vitamagatartást állít szembe: a pártfogó a saját álláspontját védi, és a másikét igyekszik elhallgattatni, a vizsgálódó pedig a vitapartnerrel közösen teszi próbára az érveket. Te az utóbbit választottad: a támadás mögötti tapasztalatból olyan kérdést csináltál, amelyet meg lehet vizsgálni. A vita tartalmasabb lesz, de időbe telik, és a párttársaid gyengeségnek láthatják.</t>
         </is>
       </c>
       <c r="H16" s="18" t="n">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="E17" s="17" t="inlineStr">
         <is>
-          <t>A menetrend a legfontosabb: lezárod a vitát, és a következő napirendi pontra lépsz, hogy a bizottság még ebben a hónapban szavazhasson.</t>
+          <t>A menetrend a legfontosabb: lezárod a vitát, és továbblépsz a következő napirendi pontra, hogy a bizottság még ebben a hónapban szavazhasson.</t>
         </is>
       </c>
       <c r="F17" s="17" t="inlineStr">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="G17" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet csoportos döntési modelljei közül az autokratikus döntésnél a vezető egyedül dönt, a tagok minimális közreműködésével. Gyors, és időhiányban indokolt lehet, de ha a tagok nem értenek egyet, a végrehajtás melletti elkötelezettségük nagyon alacsony lesz. A bizottság időben szavazhat, csak éppen kevesebbet tud arról, amiről szavaz.</t>
+          <t>A jegyzet csoportos döntési modelljei közül az autokratikus döntésnél a vezető egyedül dönt, a tagok alig vesznek részt benne. Ez gyors, és időhiányban indokolt is lehet, de ha a tagok nem értenek egyet, alig fognak elköteleződni a végrehajtás mellett. A bizottság időben szavazhat — csak éppen kevesebbet tud arról, amiről szavaz.</t>
         </is>
       </c>
       <c r="H17" s="18" t="n">
@@ -1824,12 +1824,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Három változat</t>
+          <t>Három bezárási változat</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>A bizottság asztalán három változat fekszik. Az első mind a negyven iskolát bezárja: ez a legnagyobb megtakarítás és a leghosszabb utazás. A második húszat zár be, a többiben összevont osztályok lesznek. A harmadik minden iskolát megtart, de a pénzt máshonnan kell elvenni, valószínűleg az egészségügyből. A frakció a héten döntést vár.</t>
+          <t>A bizottság asztalán három változat fekszik. Az első mind a negyven iskolát bezárná: ezzel lehetne a legtöbbet spórolni. A második húszat zárna be, a többiben összevont osztályok indulnának. A harmadik minden iskolát megtartana, de akkor máshonnan kellene elvenni a pénzt, valószínűleg az egészségügytől. A frakció még ezen a héten döntést vár.</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Nem akarsz a pártod ellen menni: a frakcióülésre bízod, melyik változatot támogassa a bizottság, te pedig levezeted a szavazást.</t>
+          <t>Nem akarsz szembemenni a pártoddal: a frakcióülésre bízod, melyik változatot támogassa a bizottság, te pedig csak levezeted a szavazást.</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>A jegyzet a döntéshozói magatartások között említi a döntés elhárítását: amikor a vezető a döntést másra hárítja, és a formális megoldást részesíti előnyben. Ez megóv a párton belüli konfliktustól, és a frakció is elégedett. Csakhogy a bizottság elnökeként épp azt a felelősséget adod ki a kezedből, amiért ott ülsz.</t>
+          <t>A jegyzet a döntéshozói magatartások között említi a döntés elhárítását: a vezető másra hárítja a döntést, és a formális megoldást választja. Ez megkímél a párton belüli konfliktustól, és a frakció is elégedett. Bizottsági elnökként azonban éppen azt a felelősséget adod ki a kezedből, amiért ott ülsz.</t>
         </is>
       </c>
       <c r="H18" s="12" t="n">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="E19" s="17" t="inlineStr">
         <is>
-          <t>A költségvetési célt teszed az első helyre: a pénzügyminisztérium ezt a számot várja, és ha a bizottság nem teljesíti, máshonnan fogják elvenni. Az első változatot támogatod.</t>
+          <t>A költségvetési célt helyezed előtérbe: a pénzügyminisztérium ezt a számot várja, és ha a bizottság nem teljesíti, máshonnan fogják elvenni a pénzt. Az első változatot támogatod.</t>
         </is>
       </c>
       <c r="F19" s="17" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="G19" s="17" t="inlineStr">
         <is>
-          <t>Simon szerint a valódi döntéshozók korlátozott racionalitással döntenek: nem mérlegelnek minden szempontot, hanem az első olyan megoldást választják, amely eléri az elvárt szintet. Itt az elvárt szint a megtakarítási cél volt, és az első változat ezt teljesíti. A döntés gyors és védhető, a többi szempont — utazás, közösség — viszont kiesett a számításból.</t>
+          <t>Simon szerint a valóságban korlátozott racionalitással döntünk: nem mérlegelünk minden szempontot, hanem az első olyan megoldást választjuk, amely eléri az elvárt szintet. Itt a megtakarítási cél volt az elvárt szint, és az első változat ezt teljesíti. A döntés gyors és védhető, a többi szempont — az utazás, a közösségek sorsa — viszont kimaradt a mérlegelésből.</t>
         </is>
       </c>
       <c r="H19" s="18" t="n">
@@ -1924,7 +1924,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="76" customHeight="1">
+    <row r="20" ht="90" customHeight="1">
       <c r="A20" s="15" t="n"/>
       <c r="B20" s="16" t="n"/>
       <c r="C20" s="17" t="n"/>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="E20" s="17" t="inlineStr">
         <is>
-          <t>Mindhárom változatnál leírod, mit nyer és mit veszít egy konkrét bükkfalvi család: hány órát utazik a gyerek, mi lesz a helyi tanítóval, mi lesz a faluval. Ezt teszed a vita középpontjába, még ha ettől érzelmesebb is lesz.</t>
+          <t>Mindhárom változatnál leírod, mit nyer és mit veszít vele egy konkrét bükkfalvi család: mennyit utazik a gyerek, mi lesz a helyi tanítóval és magával a faluval. Ezt állítod a vita középpontjába, még ha érzelmesebbé is válik tőle.</t>
         </is>
       </c>
       <c r="F20" s="17" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="G20" s="17" t="inlineStr">
         <is>
-          <t>A PrOACT-modell utolsó két lépése a következmények feltérképezése minden változatnál, és annak nyílt mérlegelése, mit adunk fel és mit kapunk érte. Egy konkrét család napjain keresztül ez a mérlegelés kézzelfoghatóvá válik. A vita emberibb lesz, de nehezebben számszerűsíthető, és a számokat váró frakciót kevésbé győzi meg.</t>
+          <t>A PrOACT-modell utolsó két lépése, hogy minden változatnál feltérképezzük a következményeket, és nyíltan mérlegeljük, mit adunk fel és mit kapunk cserébe. Egy konkrét család mindennapjain keresztül ez a mérlegelés kézzelfoghatóvá válik. A vita emberibb lesz, de nehezebben számszerűsíthető, és a számokat váró frakciót kevésbé győzi meg.</t>
         </is>
       </c>
       <c r="H20" s="18" t="n">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="E21" s="17" t="inlineStr">
         <is>
-          <t>Egymás mellé teszed a három változatot a spórolás, az utazási idő, a tanítás minősége és a falvak megtartása szerint, és először azt nézed meg, van-e köztük olyan, amelyik minden szempontból rosszabb valamelyik másiknál. Ha van, azt kihúzzátok, és csak a maradékról vitáztok. Ez alapos, de legalább egy hét.</t>
+          <t>Egymás mellé teszed a három változatot négy szempont szerint: megtakarítás, utazási idő, a tanítás minősége és a falvak megtartása. Először azt nézed meg, van-e köztük olyan, amelyik minden szempontból rosszabb valamelyik másiknál. Ha van, kihúzzátok, és csak a maradékról vitáztok. Ez alapos munka, de legalább egy hétbe telik.</t>
         </is>
       </c>
       <c r="F21" s="17" t="inlineStr">
@@ -1993,7 +1993,7 @@
       </c>
       <c r="G21" s="17" t="inlineStr">
         <is>
-          <t>A dominancia elve szerint ha egy változat semmilyen szempontból nem jobb egy másiknál, és legalább egyben rosszabb, nyugodtan kihúzhatjuk, még mielőtt bonyolult mérlegelésbe kezdenénk. Ez lecsökkenti a vitát a valóban versengő változatokra. A módszer tisztázza a választást, de az értékkérdést — mennyit ér egy falu iskolája — nem dönti el helyetted, a frakció pedig közben tovább vár.</t>
+          <t>A dominancia elve szerint ha egy változat semmilyen szempontból nem jobb egy másiknál, és legalább egyben rosszabb, nyugodtan kihúzhatjuk, még mielőtt bonyolult mérlegelésbe kezdenénk. Így a vita a valóban versengő változatokra szűkül. A módszer tisztázza a választást, de az értékkérdést — mennyit ér egy falunak az iskolája — nem dönti el helyetted, a frakció pedig közben egyre türelmetlenebb.</t>
         </is>
       </c>
       <c r="H21" s="18" t="n">
@@ -2026,12 +2026,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>A választás árnyékában</t>
+          <t>Iskolabezárás a választás előtt</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Az egyik tanácsadód egy vidéki út szélén, a következő fórumra menet kimondja, amit mindenki gondol: a megtakarítás öt év múlva jelentkezne, a választás viszont jövő tavasszal lesz, és az érintett körzetek közül hat billeg. Ha most zártok be iskolákat, ott elveszíthetitek a választást. A frakció ezt is figyeli.</t>
+          <t>A következő fórumra menet az egyik tanácsadód kimondja, amit mindenki gondol: a megtakarítás csak öt év múlva jelentkezne, a parlamenti választás viszont jövő tavasszal lesz, és az érintett körzetek közül hat billegő. Ha most zártok be iskolákat, ezekben elveszíthetitek a választást. A frakció is ezt figyeli.</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>Vállalod a menetrendet a választás előtt is, és nyilvánosan elmondod, miért: a gyerekeknek most kell a jobb iskola, nem öt év múlva. Tudod, hogy ez a pártodnak mandátumokba kerülhet.</t>
+          <t>Vállalod a menetrendet a választás előtt is, és nyilvánosan elmondod, miért: a takarékossági csomagot most kell végrehajtani. Tudod, hogy ez mandátumokba kerülhet a pártodnak.</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>A jegyzet szerint a stratégiai döntés alapvető változást indít el, és hosszú távra meghatározza a működés kereteit, míg az operatív döntés a napi működést segíti. Ha egy stratégiai döntés ütemét a választási naptár diktálja, rövid távú taktikává silányul. Te vállaltad a hosszú távot, és ki is mondtad; az ár a saját pártod bizalma és néhány körzet.</t>
+          <t>A jegyzet szerint a stratégiai döntés alapvető változást indít el, és hosszú távra kijelöli a működés kereteit, míg az operatív döntés a napi működést szolgálja. Ha egy stratégiai döntés ütemezését a választási naptár diktálja, a döntés rövid távú taktikává silányul. Te a hosszú távot vállaltad, és ezt ki is mondtad; az ára a saját pártod bizalma és néhány körzet.</t>
         </is>
       </c>
       <c r="H22" s="12" t="n">
@@ -2078,7 +2078,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="76" customHeight="1">
+    <row r="23" ht="90" customHeight="1">
       <c r="A23" s="15" t="n"/>
       <c r="B23" s="16" t="n"/>
       <c r="C23" s="17" t="n"/>
@@ -2089,7 +2089,7 @@
       </c>
       <c r="E23" s="17" t="inlineStr">
         <is>
-          <t>Kettéosztod: ahol a szülők maguk is az összevonást kérik, ott most indul, máshol két év múlva, a tapasztalatok alapján. Ez lassú és kicsit igazságtalan, de tanulhattok belőle.</t>
+          <t>Két ütemben haladtok: ahol a szülők maguk is kérik az összevonást, ott most kezditek, máshol két év múlva, a tapasztalatok alapján. Ez lassú és kissé igazságtalan, de tanulhattok belőle.</t>
         </is>
       </c>
       <c r="F23" s="17" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="G23" s="17" t="inlineStr">
         <is>
-          <t>Az inkrementalizmus a nagy, átfogó megoldások helyett kis, fokozatos lépéseket jelent, amelyekből menet közben tanulni lehet. Az önként jelentkező falvakkal kezdesz, és a tapasztalat alapján döntesz a többiről. Ez csökkenti a kockázatot, de két falu ugyanabban a helyzetben másként járhat, ami igazságtalannak tűnhet.</t>
+          <t>Az inkrementalizmus azt jelenti, hogy nagy, átfogó megoldások helyett kis, fokozatos lépésekben haladunk, és menet közben tanulunk. Az önként jelentkező falvakkal kezdesz, a többiről pedig a tapasztalatok alapján döntesz. Ez csökkenti a kockázatot, de két, ugyanolyan helyzetben lévő falu másként járhat, és ez igazságtalannak tűnhet.</t>
         </is>
       </c>
       <c r="H23" s="18" t="n">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="E24" s="17" t="inlineStr">
         <is>
-          <t>Most megszavaztatod a törvényt, de a bezárások csak a választás után indulnak. Így a döntés megszületik, a fájdalmas rész pedig később jön.</t>
+          <t>Most megszavaztatod a törvényt, de a bezárások csak a választás után kezdődnek. Így a döntés megszületik, a fájdalmas rész viszont később jön.</t>
         </is>
       </c>
       <c r="F24" s="17" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="G24" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet a döntéshozói magatartások között írja le a döntés halogatását: a problémákat sürgős és nem sürgős kategóriákba soroljuk, és kivárjuk, amíg a helyzet kikényszeríti a lépést. Formálisan döntöttél, a nehéz rész viszont a választás utánra csúszik. Ez politikailag okos, de a falvak két évig bizonytalanságban élnek, és sokan átlátnak a szitán.</t>
+          <t>A jegyzet a döntéshozói magatartások között írja le a döntés halogatását: a problémákat sürgős és nem sürgős csoportokba soroljuk, és kivárjuk, amíg a helyzet kikényszeríti a lépést. Formálisan döntöttél, a nehéz rész viszont a választás utánra tolódik. Ez politikailag okos húzás, de a falvak két évig bizonytalanságban élnek, és sokan átlátnak a szitán.</t>
         </is>
       </c>
       <c r="H24" s="18" t="n">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="E25" s="17" t="inlineStr">
         <is>
-          <t>A polgármesterekre bízod: minden falu maga dönthet az iskolájáról, és ahol megtartják, ott a kormány fizeti a különbözetet. Így senki nem mondhatja, hogy fentről döntöttek helyette — de a megtakarítás jó része elvész.</t>
+          <t>A polgármesterekre bízod a döntést: minden falu maga dönthet az iskolájáról, és ahol megtartják, ott a kormány fizeti a különbözetet. Így senki sem mondhatja, hogy a feje fölött döntöttek — a megtakarítás jó része viszont elvész.</t>
         </is>
       </c>
       <c r="F25" s="17" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg erőforrás-elosztó szerepében a vezető dönti el, hová kerül a pénz és a figyelem, és ezzel alapvetően befolyásolja mások lehetőségeit. Ezt a szerepet most kiadtad a kezedből a polgármestereknek. A döntés helyben elfogadottabb lesz, de a megtakarítási cél elveszhet, és a pénzügyminisztérium felé neked kell majd megmagyaráznod.</t>
+          <t>Mintzberg erőforrás-elosztó szerepében a vezető dönti el, hová kerül a pénz és a figyelem, és ezzel alapvetően befolyásolja mások lehetőségeit. Ezt a szerepet most kiadtad a kezedből, és átengedted a polgármestereknek. Helyben elfogadottabb lesz a döntés, de a megtakarítási cél odaveszhet, és ezt neked kell majd megmagyaráznod a pénzügyminisztériumnak.</t>
         </is>
       </c>
       <c r="H25" s="18" t="n">
@@ -2228,12 +2228,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Egyetlen szavazat</t>
+          <t>Egy szavazaton múlik</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>A bizottsági szavazás előtti estén összeszámolod: egyetlen szavazattal van meg a többség. Ekkor felhív Szalai Péter, a saját párttársad. Nemmel szavaz, hacsak le nem veszed a listáról a szülőfaluja iskoláját. Az ő faluja pontosan olyan, mint további tizenkét település a listán — csak azoknak nincs képviselőjük a bizottságban.</t>
+          <t>A bizottsági szavazás előtti estén összeszámolod a szavazatokat: egyetlen szavazaton múlik a többség. Ekkor felhív Szalai Péter, a saját párttársad: nemmel fog szavazni, hacsak le nem veszed a listáról a szülőfaluja iskoláját. Az ő faluja pontosan olyan, mint további tizenkét település a listán — csak azoknak nincs képviselőjük a bizottságban.</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Mintzberg vezető szerepe a vezető és a csapata közötti viszonyról szól: arról, milyen mércét állít fel, és azt hogyan tartja meg. Azzal, hogy a saját párttársadnak sem teszel kivételt, világossá teszed, mi érvényes a bizottságban. Ez a következetesség tiszteletet hoz, de azzal a kockázattal jár, hogy hetek munkája egyetlen szavazaton bukik el.</t>
+          <t>Mintzberg vezető szerepe a vezető és a csapata közötti viszonyról szól: milyen mércét állít fel, és hogyan tartja magát hozzá. Azzal, hogy a saját párttársadnak sem teszel kivételt, egyértelművé teszed, mi számít a bizottságban. Ez a következetesség tiszteletet szerez, de megvan a kockázata, hogy hetek munkája egyetlen szavazaton bukik el.</t>
         </is>
       </c>
       <c r="H26" s="12" t="n">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>Leveszed Szalai faluját — de ugyanazon a szempont alapján a másik tizenkét hasonló falut is. A szavazás megvan, a megtakarítás viszont a harmadával csökken, és ezt a pénzügyminisztériumnak is meg kell magyaráznod.</t>
+          <t>Leveszed a listáról Szalai faluját — de ugyanezen az alapon az összes hasonló falut is. A szavazás így átmegy, a megtakarítás viszont a harmadával csökken, és ezt a pénzügyminisztériumnak is meg kell magyaráznod.</t>
         </is>
       </c>
       <c r="F27" s="17" t="inlineStr">
@@ -2301,17 +2301,17 @@
       </c>
       <c r="G27" s="17" t="inlineStr">
         <is>
-          <t>Simon programozott döntésnek nevezi azt, amelyre előre rögzített szabály van, így minden hasonló esetben ugyanúgy születik meg. Te Szalai egyedi kérését szabállyá alakítottad, amely minden hasonló falura érvényes. Ez igazságos és védhető, de drága: kisebb a megtakarítás, és a minisztérium joggal kérdezi, miért változott a számítás az utolsó éjjel.</t>
+          <t>Simon programozott döntésnek nevezi azt, amelyre előre rögzített szabály van, így minden hasonló esetben ugyanaz a megoldás születik. Te Szalai egyéni kéréséből olyan szabályt csináltál, amely minden hasonló falura érvényes. Ez igazságos és védhető, de drága: kisebb lesz a megtakarítás, és a minisztérium joggal kérdezi, miért változott meg a számítás az utolsó éjszakán.</t>
         </is>
       </c>
       <c r="H27" s="18" t="n">
         <v>-1</v>
       </c>
       <c r="I27" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" s="18" t="n">
         <v>1</v>
@@ -2328,7 +2328,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="90" customHeight="1">
+    <row r="28" ht="104" customHeight="1">
       <c r="A28" s="15" t="n"/>
       <c r="B28" s="16" t="n"/>
       <c r="C28" s="17" t="n"/>
@@ -2339,7 +2339,7 @@
       </c>
       <c r="E28" s="17" t="inlineStr">
         <is>
-          <t>Elhalasztod a szavazást egy héttel, és addig mind a tizenhárom érintett falu polgármesterét meghallgatod, hogy lásd, kinek mennyi múlik a döntésen, és kinek mekkora a beleszólása.</t>
+          <t>Egy héttel elhalasztod a szavazást, és addig meghallgatod az összes érintett falu polgármesterét, hogy lásd, kinek mennyi múlik a döntésen, és kinek mekkora a beleszólása.</t>
         </is>
       </c>
       <c r="F28" s="17" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
-          <t>Az érintett-térkép felsorolja, kikre hat a döntés, az érintetterőtér pedig megmutatja, kinek mennyi múlik rajta és mekkora a befolyása. Szalai nagy befolyású érintett, a tizenkét másik falu viszont kiszolgáltatott helyzetben van: nagyon érinti őket a döntés, de alig van beleszólásuk. A meghallgatás kiegyensúlyozza a képet, de a csúszás a frakciót és a menetrendet is próbára teszi.</t>
+          <t>Az érintett-térkép számba veszi, kikre hat a döntés, az érintetterőtér pedig megmutatja, kinek mennyi múlik rajta, és mekkora a befolyása. Szalai nagy befolyású érintett, a tizenkét másik falu viszont kiszolgáltatott helyzetben van: őket is nagyon érinti a döntés, de alig van beleszólásuk. A meghallgatás kiegyensúlyozza a képet, de a csúszás a frakció türelmét és a menetrendet is próbára teszi.</t>
         </is>
       </c>
       <c r="H28" s="18" t="n">
@@ -2376,7 +2376,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="90" customHeight="1">
+    <row r="29" ht="104" customHeight="1">
       <c r="A29" s="15" t="n"/>
       <c r="B29" s="16" t="n"/>
       <c r="C29" s="17" t="n"/>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="E29" s="17" t="inlineStr">
         <is>
-          <t>Leveszed a listáról Szalai falujának iskoláját. A szavazás így biztosan átmegy, és a törvény — ha egy iskolával kevesebbel is — megvalósul.</t>
+          <t>Leveszed a listáról Szalai falujának iskoláját. A szavazás így biztosan átmegy, és a törvény — ha egy iskolával kevesebbre is — megvalósul.</t>
         </is>
       </c>
       <c r="F29" s="17" t="inlineStr">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="G29" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet formális moralitás detektorai közül az univerzalitás elve egyetlen kérdést tesz fel: jó lenne, ha mindenki, minden hasonló helyzetben így döntene? Ha egy falu azért marad meg, mert van képviselője a bizottságban, a tizenkét hasonló falu joggal kérdezi, nekik miért nem jár ugyanez. A szavazást megnyerted, de a szabály, amely szerint döntöttél, nem vállalható nyilvánosan.</t>
+          <t>A jegyzetben szereplő formális moralitás detektorok közül az univerzalitás elve egyetlen kérdést tesz fel: jó lenne-e, ha mindenki minden hasonló helyzetben így döntene? Ha egy falu azért tarthatja meg az iskoláját, mert van képviselője a bizottságban, a többi hasonló falu joggal kérdezi, nekik miért nem jár ugyanez. A szavazást megnyerted, de azt a szabályt, amely szerint döntöttél, nyilvánosan nem vállalhatod.</t>
         </is>
       </c>
       <c r="H29" s="18" t="n">
@@ -2430,12 +2430,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Hajnali ötkor kelni</t>
+          <t>Tüntetés a Parlament előtt</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>A javaslat — néhány módosítással — a parlament elé került. Másnap országszerte terjed egy videó: egy hétéves bükkfalvi kislány elmondja, hogy ha bezárják az iskoláját, hajnali ötkor kell majd buszra szállnia. Délutánra ezrek tüntetnek a Parlament előtt, a táblákon a te neved is ott van. A sajtó azonnali reakciót vár.</t>
+          <t>A javaslat néhány módosítással a parlament elé kerül. Másnap egy videó terjed az egész országban: egy hétéves bükkfalvi kislány elmondja, hogy ha bezárják az iskoláját, hajnali ötkor kell majd buszra szállnia. Délutánra ezrek tüntetnek a Parlament előtt, és a táblákon a te neved is szerepel. A sajtó azonnali reakciót vár tőled.</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>Felhívod a kislány családját, és megígéred, hogy az ő falujuk iskolája marad. A történet estére megfordul: a híradó már a telefonhívásodról szól.</t>
+          <t>Felhívod a kislány családját, és megígéred, hogy a falujuk iskolája megmarad. Estére megfordul a történet: a híradó már a telefonhívásodról szól.</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Az utólagossági hatás azt jelenti, hogy a legfrissebb, legélénkebb információ köré szervezzük az egész képet. A videó volt a legutolsó és legerősebb benyomás, és az egész döntést ehhez igazítottad. A gesztus emberi és gyorsan hat, de a többi falu most azt látja, hogy az számít, kinek a története kerül a híradóba.</t>
+          <t>Az utólagossági hatás azt jelenti, hogy a legfrissebb, legélénkebb információ köré rendezzük az egész képet. A videó volt a legutolsó és legerősebb benyomás, és az egész döntésedet ehhez igazítottad. A gesztus emberi, és gyorsan hat, de a többi falu most azt látja, hogy az számít, kinek a története kerül be a híradóba.</t>
         </is>
       </c>
       <c r="H30" s="12" t="n">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="E31" s="17" t="inlineStr">
         <is>
-          <t>Nem reagálsz: az ilyen hullámok két-három nap alatt elülnek, és minden nyilatkozat csak olaj a tűzre. A munkát csendben folytatod.</t>
+          <t>Nem reagálsz: az ilyen hullámok két-három nap alatt elülnek, és minden nyilatkozat csak olaj a tűzre. Csendben folytatod a munkát.</t>
         </is>
       </c>
       <c r="F31" s="17" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="G31" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet háromféle vezetői stratégiát különít el: a problémakeresőt, a problémamegoldót és a problémakerülőt, aki figyelmen kívül hagyja a valós problémahelyzeteket. A hallgatás valóban nem ad újabb muníciót a vitának, és néha a hullám tényleg elül. A tüntetők viszont azt tanulják meg, hogy a döntéshozó nem áll ki elébük, és ez a bizalomban többe kerül egy rossz nyilatkozatnál.</t>
+          <t>A jegyzet háromféle vezetői stratégiát különít el: a problémakeresőt, a problémamegoldót és a problémakerülőt, aki nem vesz tudomást a valós problémákról. A hallgatás valóban nem ad újabb muníciót a vitához, és néha a hullám tényleg magától elül. A tüntetők viszont azt szűrik le, hogy a döntéshozó nem áll ki eléjük, és ez többe kerül a bizalomban, mint egy rossz nyilatkozat.</t>
         </is>
       </c>
       <c r="H31" s="18" t="n">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="E32" s="17" t="inlineStr">
         <is>
-          <t>Közleményt adsz ki a pontos számokkal: a gyerekek átlagos utazási ideje harmincöt perc lesz, a hajnali indulás egyedi eset. A számok igazak, és nem kell kiállnod a tömeg elé.</t>
+          <t>Közleményt adsz ki a pontos számokkal: a gyerekek átlagosan harmincöt percet fognak utazni, a hajnali indulás csak egyedi eset. A számok igazak, és nem kell kiállnod a tömeg elé.</t>
         </is>
       </c>
       <c r="F32" s="17" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="G32" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet szerint a legtöbb embernél az érzelmi reakciók sokkal erősebbek a racionálisaknál: egy erős érzelmi töltetű történet mellett a pontos számok is háttérbe szorulnak. A kislány videója ilyen történet, és egy táblázat nem tud versenyezni vele. A közleményed pontos és védhető, de akik az utcán állnak, nem fogják érezni, hogy válaszoltál nekik.</t>
+          <t>A jegyzet szerint a legtöbb embernél az érzelmi reakciók jóval erősebbek a racionálisaknál: egy erős érzelmi töltetű történet mellett a pontos számok is háttérbe szorulnak. A kislány videója ilyen történet, és egy táblázat nem veheti fel vele a versenyt. A közleményed pontos és védhető, de az utcán állók nem fogják úgy érezni, hogy válaszoltál nekik.</t>
         </is>
       </c>
       <c r="H32" s="18" t="n">
@@ -2564,7 +2564,7 @@
         <v>1</v>
       </c>
       <c r="K32" s="18" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="L32" s="18" t="n">
         <v>-2</v>
@@ -2589,7 +2589,7 @@
       </c>
       <c r="E33" s="17" t="inlineStr">
         <is>
-          <t>Kimész a tüntetők közé, és elmondod, mit vállalsz és mit nem: a hajnali indulást megakadályozod, de az összevonásokat nem vonod vissza. Tudod, hogy kifütyülhetnek, és minden szavadat felveszik.</t>
+          <t>Kimész a tüntetők közé, és elmondod, mit vállalsz és mit nem: a hajnali indulást nem engeded, de az összevonásokat nem vonod vissza. Tudod, hogy kifütyülhetnek, és minden szavadat felveszik.</t>
         </is>
       </c>
       <c r="F33" s="17" t="inlineStr">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="G33" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg szóvivő szerepében a vezető a kívülállóknak adja át az információt: elmondja, mit tesznek és miért. Személyesen, a tüntetők előtt vállalni egy kényelmetlen üzenetet ennek a legnehezebb és leghitelesebb formája. Ugyanakkor minden mondatod kötelezettség lesz, amelyet később számon kérnek rajtad.</t>
+          <t>Mintzberg szóvivő szerepében a vezető a kívülállókat tájékoztatja: elmondja, mit tesznek és miért. Ennek a legnehezebb és leghitelesebb formája, ha személyesen, a tüntetők előtt vállalsz egy kényelmetlen üzenetet. Ugyanakkor minden mondatod kötelezettséggé válik, amelyet később számon kérnek rajtad.</t>
         </is>
       </c>
       <c r="H33" s="18" t="n">
@@ -2632,12 +2632,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>A tanulmány</t>
+          <t>A kedvezőtlen tanulmány</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>A parlamenti zárószavazás reggelén egy minisztériumi munkatárs átad neked egy belső tanulmányt. Eszerint a megtakarítás negyven százalékkal kisebb lesz a tervezettnél, mert a buszok és a városi iskolák bővítése többe kerül. A tanulmány még nem végleges, és rajtad kívül alig néhányan látták. Két óra múlva kezdődik a vita, amelyet te nyitsz meg.</t>
+          <t>A parlamenti zárószavazás reggelén egy minisztériumi munkatárs átad neked egy belső tanulmányt. Eszerint a megtakarítás negyven százalékkal kisebb lesz a tervezettnél, mert a buszok és a városi iskolák bővítése többe kerül. A tanulmány még nem végleges, és rajtad kívül csak néhányan látták. Két óra múlva kezdődik a vita, és te nyitod meg.</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>Megszavazzátok a törvényt, de beteszel egy záradékot: két év múlva független felülvizsgálat jön, és ha a megtakarítás nem teljesül, a további bezárásokat felfüggesztik.</t>
+          <t>Megszavazzátok a törvényt, de beteszel egy záradékot: két év múlva független felülvizsgálatot tartanak, és ha a megtakarítás elmarad, a további bezárásokat felfüggesztik.</t>
         </is>
       </c>
       <c r="F34" s="11" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Snowden és Boone szerint komplex helyzetben nincs előre ismert helyes válasz: az okok és hatások csak menet közben derülnek ki, ezért a jó vezető kísérletezik, figyel, és kész korrigálni. A záradékkal ezt a tanulási lehetőséget építetted be a törvénybe. A megoldás bölcs, de félmegoldásnak is látszhat: a tanulmányt nem hoztad nyilvánosságra, és a bezárások egy része akkor is megtörténik, ha a számok rosszak.</t>
+          <t>Snowden és Boone szerint komplex helyzetben nincs előre ismert helyes válasz: az okok és a hatások csak menet közben derülnek ki, ezért a jó vezető kísérletezik, figyel, és kész korrigálni. A záradékkal ezt a tanulási lehetőséget építetted be a törvénybe. Bölcs megoldás, de félmegoldásnak is tűnhet: a tanulmányt nem hoztad nyilvánosságra, és a bezárások egy része akkor is megtörténik, ha a számok rosszak.</t>
         </is>
       </c>
       <c r="H34" s="12" t="n">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="E35" s="17" t="inlineStr">
         <is>
-          <t>Nem említed: a tanulmány nem végleges, a törvény mellett a megtakarításon kívül is vannak érvek, és egy félkész szám most csak zavart keltene.</t>
+          <t>Nem említed: a tanulmány nem végleges, a törvény mellett a megtakarításon kívül is szólnak érvek, és egy félkész szám most csak zavart keltene.</t>
         </is>
       </c>
       <c r="F35" s="17" t="inlineStr">
@@ -2705,7 +2705,7 @@
       </c>
       <c r="G35" s="17" t="inlineStr">
         <is>
-          <t>A szelektív hárítás az, amikor a kellemetlen, a kialakult képbe nem illő információt nem engedjük be. Az érvelésed nem légből kapott: a tanulmány tényleg nem végleges. Ha viszont a számok később igaznak bizonyulnak, nem az lesz a kérdés, mit tudtál, hanem az, hogy miért hallgattál.</t>
+          <t>Szelektív hárításról akkor beszélünk, amikor a kellemetlen, a kialakult képbe nem illő információt nem engedjük be. Az érvelésed nem alaptalan: a tanulmány valóban nem végleges. Ha azonban a számok később beigazolódnak, nem az lesz a kérdés, mit tudtál, hanem az, hogy miért hallgattál.</t>
         </is>
       </c>
       <c r="H35" s="18" t="n">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E36" s="17" t="inlineStr">
         <is>
-          <t>Megkéred a minisztert, hogy a szavazás előtt hivatalosan erősítse meg vagy cáfolja a számokat. Ha nem teszi, a minisztérium hivatalos adataira támaszkodva igennel szavazol.</t>
+          <t>Megkéred a minisztert, hogy a szavazás előtt hivatalosan erősítse meg vagy cáfolja a számokat. Ha nem teszi meg, a minisztérium hivatalos adataira támaszkodva igennel szavazol.</t>
         </is>
       </c>
       <c r="F36" s="17" t="inlineStr">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="G36" s="17" t="inlineStr">
         <is>
-          <t>Az ezredes-hatás az a hajlamunk, hogy a magas beosztású emberektől érkező információt hitelesebbnek tartjuk. Ha a miniszter hallgat, az ő hallgatását fogadod el végső szónak, pedig a tanulmány ugyanabból a minisztériumból jött. Ez formálisan védhető, de a döntés felelősségét valaki másra helyezed át.</t>
+          <t>Az ezredes-hatás az a hajlamunk, hogy a magas beosztású emberektől érkező információt hitelesebbnek tartjuk. Ha a miniszter hallgat, az ő hallgatását fogadod el végső szónak, pedig a tanulmány ugyanabból a minisztériumból származik. Ez formálisan védhető, de a döntés felelősségét másra hárítod.</t>
         </is>
       </c>
       <c r="H36" s="18" t="n">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="G37" s="17" t="inlineStr">
         <is>
-          <t>Drucker hatékony döntéshozatali lépései közül az utolsó az, hogy a döntés érvényességét folyamatosan teszteljük a friss események tükrében: jók-e még az előfeltevéseink? A tanulmány éppen ilyen friss esemény, és te nem tetted félre. Ez szakmailag tisztességes lépés, de politikailag súlyos ára van, és a halasztás alatt a falvak bizonytalanságban maradnak.</t>
+          <t>Drucker hatékony döntéshozatali lépései közül az utolsó az, hogy a döntés érvényességét az újabb események fényében folyamatosan ellenőrizzük: megállják-e még a helyüket a kiinduló feltevéseink? A tanulmány éppen ilyen új fejlemény, és te nem söpörted le az asztalról. Szakmailag ez tisztességes lépés, de politikailag súlyos ára van, és a halasztás alatt a falvak bizonytalanságban maradnak.</t>
         </is>
       </c>
       <c r="H37" s="18" t="n">
@@ -2834,12 +2834,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Levél Bükkfalváról</t>
+          <t>Számvetés a szavazás után</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>A szavazás lezajlott. Este egyedül ülsz az irodádban. Az asztalodon egy kézzel írt levél a bükkfalvi kislánytól, mellette egy riporter üzenete: holnap reggel interjút kér, és egyetlen kérdése lesz — mit tanultál ebből a tíz hétből? Most kell eldöntened, mit mondasz, és mit kezdesz a tapasztalattal.</t>
+          <t>A szavazás lezajlott. Este egyedül ülsz az irodádban. Az asztalodon egy kézzel írt levél a bükkfalvi kislánytól, mellette egy riporter üzenete: holnap reggel interjút kér, és az egyik kérdését előre megírja — mit tanultál ebből a tíz hétből? Most kell eldöntened, mit mondasz, és mit kezdesz a tapasztalataiddal.</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
@@ -2849,7 +2849,7 @@
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>Azt mondod: a költségvetés, a párt és a határidő nem hagyott más utat, és a lehető legjobbat hoztad ki belőle. Ez nagyrészt igaz is.</t>
+          <t>Azt mondod, hogy a költségvetés, a párt és a határidő nem hagyott más utat, és te kihoztad belőle a lehető legjobbat.</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Az énmegerősítő attribúció az a hajlamunk, hogy a sikereinket magunknak, a kudarcainkat pedig a körülményeknek tulajdonítsuk. Nem hazudsz: a körülmények valóban szorítottak. Ha viszont csak ezt látod, éppen azt a részt hagyod ki, amelyből tanulni lehetne — a saját döntéseidet.</t>
+          <t>Az énmegerősítő attribúció az a hajlamunk, hogy a sikereinket magunknak, a kudarcainkat pedig a körülményeknek tulajdonítjuk. Nem hazudsz: a körülmények valóban szorítottak. Ha viszont csak ezt látod, éppen azt hagyod ki, amiből tanulni lehetne: a saját döntéseidet.</t>
         </is>
       </c>
       <c r="H38" s="12" t="n">
@@ -2897,7 +2897,7 @@
       </c>
       <c r="E39" s="17" t="inlineStr">
         <is>
-          <t>Nem adsz interjút. Úgy gondolod, a számok és az idő majd igazolnak, és felesleges most magyarázkodni.</t>
+          <t>Nem adsz interjút. Úgy gondolod, a számok és az idő majd igazolnak, és fölösleges most magyarázkodni.</t>
         </is>
       </c>
       <c r="F39" s="17" t="inlineStr">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="G39" s="17" t="inlineStr">
         <is>
-          <t>James March hamisan pozitív hibának nevezi, amikor a döntéshozó komolyan hisz egy olyan kontrollban, amely a valóságban nincs meg. Abban bízni, hogy az idő magától igazol, ilyen hit: a számok értelmezése nem a te kezedben lesz. A hallgatás megóv egy nehéz beszélgetéstől, de a kérdést nyitva hagyja, és mások fogják megválaszolni helyetted.</t>
+          <t>James March hamisan pozitív hibának nevezi, amikor a döntéshozó szentül hisz egy olyan kontrollban, amely a valóságban nincs a kezében. Az a meggyőződés, hogy az idő majd magától igazol, ilyen hit: a számok értelmezése nem rajtad fog múlni. A hallgatás megkímél egy nehéz beszélgetéstől, de nyitva hagyja a kérdést, és mások fognak válaszolni helyetted.</t>
         </is>
       </c>
       <c r="H39" s="18" t="n">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="G40" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet szerint a csoportos döntések során megoszlik a felelősség, a valóban bevont résztvevők pedig elkötelezettebbé válnak. Egy közös visszatekintés több nézőpontot hoz, mint a te egyedüli mérlegelésed. Az ára, hogy a saját felelősséged beleolvad a közösbe, és a jelentés óvatosabb lesz egy személyes vallomásnál.</t>
+          <t>A jegyzet szerint csoportos döntésnél megoszlik a felelősség, a valóban bevont résztvevők pedig jobban elköteleződnek. Egy közös visszatekintés több nézőpontot hoz, mint ha egyedül mérlegelnél. Az ára, hogy a saját felelősséged feloldódik a közösben, és a jelentés óvatosabb lesz egy személyes vallomásnál.</t>
         </is>
       </c>
       <c r="H40" s="18" t="n">
@@ -2982,7 +2982,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="76" customHeight="1">
+    <row r="41" ht="90" customHeight="1">
       <c r="A41" s="15" t="n"/>
       <c r="B41" s="16" t="n"/>
       <c r="C41" s="17" t="n"/>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="G41" s="17" t="inlineStr">
         <is>
-          <t>A következtetési létra azt írja le, hogyan jutunk a látott tényekből villámgyorsan feltevésekhez és ítéletekhez; a reflektív gondolkodás ezen a létrán való tudatos lemászás. Ha végigveszed, melyik feltevésed vezetett félre, a következő döntésed jobb lesz. A nyilvános beismerés hiteles, de politikailag sebezhetővé tesz.</t>
+          <t>A következtetési létra azt írja le, hogyan jutunk el villámgyorsan a látott tényektől a feltevésekig és az ítéletekig; a reflektív gondolkodás azt jelenti, hogy tudatosan visszamászunk ezen a létrán. Ha végiggondolod, melyik feltevésed vezetett félre, legközelebb jobban fogsz dönteni. A nyilvános beismerés hiteles, de politikailag sebezhetővé tesz.</t>
         </is>
       </c>
       <c r="H41" s="18" t="n">
@@ -3191,12 +3191,12 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>Péntekre egy terv</t>
+          <t>Válságterv péntekre</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Hétfő reggel levelet kapsz a vezérigazgatótól: a patikalánc felmondással fenyeget, pénteken tervet kér tőled. Réka, a patikalánccal foglalkozó csapat vezetője már délelőtt bejön egy kész ötlettel: vegyetek fel tíz ideiglenes munkatársat, és péntekre a terv is kész. A csapat kimerült, a vezérigazgató türelmetlen.</t>
+          <t>Hétfő reggel a vezérigazgató péntekre válságtervet kér tőled, mert a legnagyobb ügyfeletek, egy patikalánc, fel akarja mondani a szerződést. Réka, a patikaláncért felelős csapat vezetője rögtön elő is áll egy mentőötlettel: vegyetek fel tíz ideiglenes munkatársat. A vezetés türelmetlen, a csapat a teherbírása határán van, tíz új ember betanítása pedig komoly kockázat.</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>Elfogadod Réka ötletét: tíz ideiglenes munkatárs, péntekre kész a terv. Gyors, érthető, és a csapat is megkönnyebbül.</t>
+          <t>Elfogadod Réka ötletét: tíz ideiglenes munkatárs, és péntekre kész a terv. Gyors, érthető megoldás, és a csapat is megkönnyebbül.</t>
         </is>
       </c>
       <c r="F2" s="11" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Simon programozott döntésnek nevezi azt, amelyre kész rutin van, nem programozottnak azt, amelyre nincs előírt és követhető út. A „több ember kell” bevett válasz egy olyan helyzetre, amelyet még senki nem értett meg igazán. Gyorsan cselekszel, és a csapat hálás, de ha a baj nem a létszámban van, tíz új ember csak több hibát fog termelni.</t>
+          <t>Simon programozott döntésnek nevezi azt, amelyre van kész rutin, nem programozottnak pedig azt, amelyre nincs előírt, követhető út. A „több ember kell” bevett válasz egy olyan helyzetre, amelyet még senki sem értett meg igazán. Gyorsan lépsz, és a csapat hálás érte, de ha a baj nem a létszámmal van, tíz új ember csak még több hibát fog okozni.</t>
         </is>
       </c>
       <c r="H2" s="12" t="n">
@@ -3254,7 +3254,7 @@
       </c>
       <c r="E3" s="17" t="inlineStr">
         <is>
-          <t>Pénteken egy nagy átalakítási tervet teszel le: új rendszer, új folyamatok, új csapatbeosztás, mindent egyszerre. A vezérigazgató lenyűgözve lesz, de a csapat nem tudja, hogyan bírja majd.</t>
+          <t>Pénteken egy átfogó átalakítási tervet teszel le az asztalra: új rendszer, új folyamatok, új csapatbeosztás, mindez egyszerre. A vezérigazgatót lenyűgözi, a csapat viszont nem tudja, hogyan fogja bírni.</t>
         </is>
       </c>
       <c r="F3" s="17" t="inlineStr">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
-          <t>Snowden és Boone szerint egyszerű helyzetben ismert a helyes válasz, komplex helyzetben viszont az okok és hatások csak menet közben derülnek ki, ezért óvatosan, kis lépésekben kell haladni. A nagy terv úgy kezeli a helyzetet, mintha már tudnád a választ. Felülről erősnek látszol, alulról viszont egy kimerült csapatra teszel még egy terhet.</t>
+          <t>Snowden és Boone szerint egyszerű helyzetben ismert a helyes válasz, komplex helyzetben viszont az okok és a hatások csak menet közben derülnek ki, ezért óvatosan, kis lépésekben kell haladni. A nagy terv úgy kezeli a helyzetet, mintha már tudnád a választ. Felülről nézve erősnek tűnsz, de egy kimerült csapatra raksz még egy terhet.</t>
         </is>
       </c>
       <c r="H3" s="18" t="n">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="E4" s="17" t="inlineStr">
         <is>
-          <t>Még aznap felhívod a patikalánc beszerzési vezetőjét, és megkérdezed, mi zavarja őket leginkább. Tudod, hogy a vezérigazgató nem szereti, ha az ő tudta nélkül tárgyalsz az ügyféllel.</t>
+          <t>Még aznap felhívod a patikalánc beszerzési vezetőjét, és megkérdezed, mi zavarja őket a leginkább. Tudod, hogy a vezérigazgató nem szereti, ha a tudta nélkül tárgyalsz az ügyféllel.</t>
         </is>
       </c>
       <c r="F4" s="17" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="G4" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg kapcsolattartó szerepében a vezető kapcsolatot tart a szervezeten kívüliekkel, és ezen keresztül olyan információhoz jut, amely bentről nem látszik. Az ügyfél szavaiból pontosabb képet kapsz, mint bármilyen belső riportból. A hívás viszont a vezérigazgató feje fölött történt, és ezt ő is így fogja látni.</t>
+          <t>Mintzberg kapcsolattartó szerepében a vezető a szervezeten kívüliekkel tartja a kapcsolatot, és így olyan információhoz jut, amely belülről nem látszik. Az ügyfél szavaiból pontosabb képet kapsz, mint bármilyen belső jelentésből. A hívás viszont a vezérigazgató feje fölött történt, és ő is így fogja látni.</t>
         </is>
       </c>
       <c r="H4" s="18" t="n">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="E5" s="17" t="inlineStr">
         <is>
-          <t>Csütörtökig nem írsz tervet: előbb leülsz Rékával és a két legtapasztaltabb ügyintézővel, és leírjátok, mi pontosan a baj, mit akar a patikalánc, és mit nem szeretnétek feláldozni. A vezérigazgató így csak az utolsó pillanatban kap anyagot.</t>
+          <t>Csütörtökig nem írsz tervet: előbb leülsz Rékával és a két legtapasztaltabb ügyintézővel, és leírjátok, pontosan mi a baj, mit akar a patikalánc, és mit nem akartok feláldozni. Így a vezérigazgató csak az utolsó pillanatban kap anyagot.</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
-          <t>Ez a PrOACT-modell eleje: a probléma pontos meghatározása és a célok összegyűjtése, mielőtt bármilyen megoldásról döntenénk. Réka ötlete már egy kész válasz volt, te viszont előbb azt tisztáztad, mi a kérdés. Ennek ára a feszes határidő és egy vezérigazgató, aki addig nem lát semmit.</t>
+          <t>Ez a PrOACT-modell eleje: pontosan meghatározni a problémát és összegyűjteni a célokat, mielőtt bármilyen megoldásról döntenénk. Réka ötlete már kész válasz volt, te viszont előbb azt tisztáztad, mi a kérdés. Ennek ára a szoros határidő és egy vezérigazgató, aki addig semmit sem lát.</t>
         </is>
       </c>
       <c r="H5" s="18" t="n">
@@ -3387,18 +3387,18 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="76" customHeight="1">
+    <row r="6" ht="90" customHeight="1">
       <c r="A6" s="9" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Egymást hibáztatják</t>
+          <t>Egymást hibáztató osztályok</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Szerdán összehívod az érintett vezetőket. Gábor, az értékesítési igazgató szerint a baj az, hogy az üzemeltetés lassú. Anita, az üzemeltetés vezetője szerint az értékesítés lehetetlen határidőket ígér. A raktár és az informatika képviselője hallgat. Egy órád van, és a végén mindenki azt várja, hogy te mondd meg, hol a hiba.</t>
+          <t>Szerdára összehívod az érintett vezetőket. Gábor, az értékesítési igazgató szerint az a baj, hogy lassú az üzemeltetés. Anita, az üzemeltetés vezetője szerint az értékesítés teljesíthetetlen határidőket ígér. A raktár és az informatika képviselője hallgat. Egy órád van, és a végén mindenki azt várja, hogy te mondd meg, hol a hiba.</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>A táblára felírjátok, kiket érint a patikalánc kiszolgálása — értékesítés, üzemeltetés, raktár, informatika, a patikusok, sőt a betegek is —, és mindegyiknél azt, mennyi múlik rajtuk és mekkora a beleszólásuk. Az óra végére még nincs döntés.</t>
+          <t>Felírjátok a táblára, kiket érint a patikalánc kiszolgálása — az értékesítést, az üzemeltetést, a raktárt, az informatikát, a patikusokat, sőt a betegeket is —, és mindegyiknél azt, mennyi múlik rajtuk, és mekkora a beleszólásuk. Az óra végére még nincs döntés.</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Az érintett-térkép azt mutatja meg, kik mind érintettek egy döntésben, beleértve azokat is, akik nincsenek a teremben, például a patikusokat és a betegeket. Ettől a vita a hibáztatásról átkerült arra, kinek mi a dolga. Az ára, hogy az óra végén még nincs döntés, és Gábor ezt időhúzásnak fogja látni.</t>
+          <t>Az érintett-térkép megmutatja, kiket érint egy döntés, azokat is beleértve, akik nem ülnek a teremben, például a patikusokat és a betegeket. Ettől a vita a hibáztatás helyett arra terelődött, kinek mi a dolga. Az ára, hogy az óra végén még nincs döntés, és Gábor ezt időhúzásnak fogja látni.</t>
         </is>
       </c>
       <c r="H6" s="12" t="n">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="E7" s="17" t="inlineStr">
         <is>
-          <t>Megkérsz minden területet, hogy péntekig írja le, szerinte mi a baj, és ezeket összesíted. Mindenki szót kap, de tudod, hogy öt különböző választ fogsz kapni.</t>
+          <t>Megkéred mindegyik területet, hogy péntekig írja le, szerinte mi a baj, és ezeket összesíted. Mindenki szóhoz jut, de tudod, hogy öt különböző választ fogsz kapni.</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>A szelektív észlelés az, amikor mindenki abból a szemszögből látja a problémát, ahonnan jön: a jegyzet példájában a marketinges a reklámban, a pénzügyes a pénzügyekben látja a bajt. Minden terület a saját válaszát fogja hozni, és ezeket egymás mellé tenni már önmagában tanulságos. A kép viszont széttöredezett marad, és a döntés terhe továbbra is rajtad lesz.</t>
+          <t>Szelektív észlelésről akkor beszélünk, amikor mindenki a saját szemszögéből látja a problémát: a jegyzet példájában a marketinges a reklámban, a pénzügyes a pénzügyekben keresi a bajt. Minden terület a saját válaszát fogja hozni, és már az is tanulságos, ha ezeket egymás mellé teszed. A kép viszont széttöredezett marad, és a döntés terhe továbbra is a te válladat nyomja.</t>
         </is>
       </c>
       <c r="H7" s="18" t="n">
@@ -3504,7 +3504,7 @@
       </c>
       <c r="E8" s="17" t="inlineStr">
         <is>
-          <t>Nem engeded tovább a vitát: a múlt heti tájékoztatón azt hallottad, hogy a raktár késik, ezért kimondod, hogy a gond ott van, és oda küldesz erősítést. Legalább történik valami.</t>
+          <t>Nem hagyod tovább folyni a vitát: a múlt heti tájékoztatón azt hallottad, hogy a raktár késik, ezért kimondod, hogy ott van a gond, és oda küldesz erősítést. Legalább történik valami.</t>
         </is>
       </c>
       <c r="F8" s="17" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>Az elsőségi hatás azt jelenti, hogy a legelső információ köré szervezzük a később kapottakat: az első benyomás határozza meg az egész képet. A raktárról hallott első hír lett a kiindulópontod, és az egész vitát ehhez igazítottad. Ez gyors és határozott lépés, de ha az első hír félrevezetett, most rossz helyre küldesz embert.</t>
+          <t>Az elsőségi hatás azt jelenti, hogy a legelső információ köré rendezzük a később kapottakat: az első benyomás határozza meg az egész képet. A raktárról hallott első hír lett a kiindulópontod, és az egész vitát ehhez igazítottad. Gyors és határozott lépés, de ha az első hír félrevezető volt, most rossz helyre küldesz embert.</t>
         </is>
       </c>
       <c r="H8" s="18" t="n">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="E9" s="17" t="inlineStr">
         <is>
-          <t>Gábornak adsz igazat: az üzemeltetésről mindenki tudja, hogy lassú és merev, az értékesítés pedig hozza a pénzt. Anita elsápad, de a vita gyorsan lezárul.</t>
+          <t>Gábornak adsz igazat: mindenki tudja, hogy az üzemeltetés lassú és merev, az értékesítés pedig hozza a pénzt. Anita elsápad, de a vita gyorsan lezárul.</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">
@@ -3562,7 +3562,7 @@
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>A sztereotipizálás az, amikor valakit az alapján ítélünk meg, ahogyan azt a csoportot látjuk, amelyhez tartozik. Az „üzemeltetés lassú” kép kényelmes és gyors, és néha igaz is. Itt viszont eldöntötted a kérdést anélkül, hogy megnézted volna, tényleg ott van-e a baj — és Anita csapata ezt nem fogja elfelejteni.</t>
+          <t>Sztereotipizálásról akkor beszélünk, amikor valakit aszerint ítélünk meg, hogyan látjuk azt a csoportot, amelyhez tartozik. A „lassú üzemeltetés” képe kényelmes és gyors, és néha igaz is. Itt viszont úgy döntöttél, hogy meg sem nézted, tényleg ott van-e a baj — és ezt Anita csapata nem fogja elfelejteni.</t>
         </is>
       </c>
       <c r="H9" s="18" t="n">
@@ -3589,18 +3589,18 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="76" customHeight="1">
+    <row r="10" ht="90" customHeight="1">
       <c r="A10" s="9" t="n">
         <v>3</v>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>„Cseréld le Rékát”</t>
+          <t>Nyomás Réka leváltására</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>A vezérigazgató behív az irodájába. A tulajdonosok nyugtalanok, és szerinte a gond Réka: ő vezeti a patikalánc-csapatot, nála csúsznak a dolgok. Azt mondja, cseréld le. Te tudod, hogy Réka csapatához tavasz óta harminc százalékkal több ügy érkezik, ugyanannyi emberrel.</t>
+          <t>A vezérigazgató behív az irodájába. A tulajdonosok nyugtalanok, és szerinte Réka a gond: ő vezeti a patikalánccal foglalkozó csapatot, és nála csúsznak a dolgok. Azt kéri, hogy cseréld le. Te viszont tudod, hogy Réka csapatához tavasz óta harminc százalékkal több ügy érkezik, ugyanannyi emberrel.</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Az alapvető attribúciós hiba az a hajlamunk, hogy mások kudarcát a személyükkel magyarázzuk, és alábecsüljük a helyzet hatását. Réka csapatának harminc százalékkal több munkája lett, a döntés mégis őt nevezte meg okként. A leváltás gyors jel a tulajdonosoknak, de ha a terhelés marad, az új vezető ugyanígy fog elbukni.</t>
+          <t>Az alapvető attribúciós hiba az a hajlamunk, hogy mások kudarcát a személyükkel magyarázzuk, a helyzet hatását pedig alábecsüljük. Réka csapatának harminc százalékkal több munkája lett, a döntés mégis őt nevezte meg okként. A leváltás gyors jelzés a tulajdonosoknak, de ha a terhelés nem csökken, az új vezető ugyanígy el fog bukni.</t>
         </is>
       </c>
       <c r="H10" s="12" t="n">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="E11" s="17" t="inlineStr">
         <is>
-          <t>Kiállsz Réka mellett, és megmutatod a vezérigazgatónak a számokat: a csapata terhelése harminc százalékkal nőtt. Tudod, hogy ha a helyzet nem javul, innentől te is a célkeresztbe kerülsz.</t>
+          <t>Kiállsz Réka mellett, és megmutatod a vezérigazgatónak a számokat: a csapata terhelése harminc százalékkal nőtt. Tudod, hogy ha a helyzet nem javul, innentől te is célkeresztbe kerülsz.</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg vezető szerepe a vezető és a beosztottai közötti viszonyról szól, és ez hatja át az egész vezetői munkát. Azzal, hogy nyomás alatt is kiálltál Réka mellett, a csapat azt látja, hogy számíthat rád. Ezzel viszont a saját hitelességedet is odatetted mellé: ha a számok nem javulnak, a kérdés már rólad fog szólni.</t>
+          <t>Mintzberg vezető szerepe a vezető és a beosztottai közötti viszonyról szól, és ez az egész vezetői munkát áthatja. Azzal, hogy nyomás alatt is kiálltál Réka mellett, a csapat azt látja, hogy számíthat rád. Ezzel viszont a saját hitelességedet is kockára tetted: ha a számok nem javulnak, a kérdés már rólad fog szólni.</t>
         </is>
       </c>
       <c r="H11" s="18" t="n">
@@ -3716,7 +3716,7 @@
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>Az önbeteljesítő jóslat — más néven Pygmalion-hatás — azt jelenti, hogy amit valakiről elvárunk, az a viselkedésünkön keresztül valóra is válik. Ha Réka érzi, hogy gyengének tartják, nagy eséllyel bizonytalanabbul és rosszabbul fog dolgozni. A kompromisszum mindenkit megnyugtat egy időre, de éppen azt a teljesítményt rontja, amelyet javítani akartál.</t>
+          <t>Az önbeteljesítő jóslat — más néven Pygmalion-hatás — azt jelenti, hogy amit valakitől elvárunk, az a saját viselkedésünk révén valóra is válik. Ha Réka érzi, hogy gyengének tartják, nagy eséllyel bizonytalanabbul és rosszabbul fog dolgozni. A kompromisszum egy időre mindenkit megnyugtat, de éppen azt a teljesítményt rontja, amelyen javítani akartál.</t>
         </is>
       </c>
       <c r="H12" s="18" t="n">
@@ -3754,7 +3754,7 @@
       </c>
       <c r="E13" s="17" t="inlineStr">
         <is>
-          <t>Azt mondod a vezérigazgatónak, hogy két hét múlva adatokkal jössz vissza, és addig semmihez nem nyúlsz. Ő ezt nem szívesen hallja, de beleegyezik.</t>
+          <t>Azt mondod a vezérigazgatónak, hogy két hét múlva adatokkal jössz vissza, addig pedig semmihez sem nyúlsz. Nem szívesen hallja, de beleegyezik.</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>Herbert Simon szerint a döntés három lépésből áll: megértés, tervezés, választás. A megértés a helyzetről szóló tudás összegyűjtését és rendezését jelenti, még a lehetőségek kidolgozása előtt. Két hetet nyertél arra, hogy tények alapján dönts Rékáról, de a vezérigazgató türelme véges, és a csapat addig bizonytalanságban dolgozik.</t>
+          <t>Herbert Simon szerint a döntés három szakaszból áll: megértés, tervezés, választás. A megértés azt jelenti, hogy összegyűjtjük és rendszerezzük a helyzetről szóló tudást, még mielőtt kidolgoznánk a lehetőségeket. Két hetet nyertél arra, hogy tények alapján dönts Rékáról, de a vezérigazgató türelme véges, és a csapat addig bizonytalanságban dolgozik.</t>
         </is>
       </c>
       <c r="H13" s="18" t="n">
@@ -3797,12 +3797,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Az aznapi ígéret</t>
+          <t>Teljesíthetetlen szállítási ígéretek</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Kiderül, hogy a hibák jó része abból fakad, hogy az értékesítés aznapi szállítást ígér a patikáknak, amit az üzemeltetés nem tud tartani. Csakhogy az értékesítők prémiuma éppen ezektől a megrendelésektől függ. Anita szabályt akar, Gábor azzal fenyeget, hogy a vezérigazgatóhoz megy.</t>
+          <t>Kiderül, hogy a hibák jó része abból fakad, hogy az értékesítés aznapi szállítást ígér a patikáknak, amit az üzemeltetés nem tud teljesíteni. Csakhogy az értékesítők prémiuma éppen ezektől a megrendelésektől függ. Anita szabályozást akar, Gábor pedig azzal fenyeget, hogy a vezérigazgatóhoz fordul.</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
@@ -3812,7 +3812,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Úgy döntesz, ez a két osztályvezető ügye: egyezzenek meg ők, te nem szólsz bele. Így senki nem mondhatja, hogy elfogult vagy.</t>
+          <t>Úgy döntesz, hogy ez a két osztályvezető ügye: egyezzenek meg egymással, te nem szólsz bele. Így senki sem mondhatja, hogy elfogult vagy.</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
@@ -3822,7 +3822,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>A jegyzet a döntéshozói magatartások között írja le a döntés elhárítását: a vezető másokra hagyja a döntést, és a formális megoldást részesíti előnyben. Kívülről semlegesnek tűnsz, de a két osztályvezető között éppen az hiányzik, aki el tudná dönteni a vitát. A konfliktus valószínűleg a vezérigazgató asztalán köt ki — nélküled.</t>
+          <t>A jegyzet a döntéshozói magatartások között írja le a döntés elhárítását: a vezető másokra hagyja a döntést, és a formális megoldást választja. Kívülről semlegesnek tűnsz, de a két osztályvezető vitájából éppen az hiányzik, aki dönteni tudna. A konfliktus valószínűleg a vezérigazgató asztalán köt ki — nélküled.</t>
         </is>
       </c>
       <c r="H14" s="12" t="n">
@@ -3860,7 +3860,7 @@
       </c>
       <c r="E15" s="17" t="inlineStr">
         <is>
-          <t>Közös megbeszélést tartasz az értékesítőkkel és az üzemeltetőkkel, ahol ők maguk rakják össze, mit lehet megígérni és mit nem. A szabály az övék lesz, de legalább két hétig tart.</t>
+          <t>Közös megbeszélést tartasz az értékesítőknek és az üzemeltetőknek, ahol ők maguk dolgozzák ki, mit lehet megígérni és mit nem. A szabály az övék lesz, de legalább két hétbe telik.</t>
         </is>
       </c>
       <c r="F15" s="17" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>A részvételi létra azt mutatja, mennyire valódi a bevonás: puszta tájékoztatás, meghallgatás vagy tényleges döntési jog. Te a létra felső fokán jártál, a szabályt az érintettek maguk alakítják ki. Ettől jobban be is tartják majd, de két hétig a régi gyakorlat fut tovább, és a patikalánc közben nem vár.</t>
+          <t>A részvételi létra azt mutatja meg, mennyire valódi a bevonás: puszta tájékoztatás, meghallgatás vagy tényleges döntési jog. Te a létra felső fokára léptél: a szabályt maguk az érintettek alakítják ki. Ezért jobban be is fogják tartani, de két hétig a régi gyakorlat megy tovább, a patikalánc pedig közben nem vár.</t>
         </is>
       </c>
       <c r="H15" s="18" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="E16" s="17" t="inlineStr">
         <is>
-          <t>Megtartjátok az aznapi ígéretet, de az üzemeltetés kap három új embert, akiket az értékesítési prémiumkeretből fizettek. A szállítás tartható lesz, Gábor viszont dühös, mert az ő csapata fizeti a számlát.</t>
+          <t>Megmarad az aznapi szállítás ígérete, de az üzemeltetés kap három új embert, akiket az értékesítési prémiumkeretből fizettek. A szállítás így tartható lesz, Gábor viszont dühös, mert az ő csapata állja a számlát.</t>
         </is>
       </c>
       <c r="F16" s="17" t="inlineStr">
@@ -3918,7 +3918,7 @@
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg erőforrás-elosztó szerepében a vezető dönti el, hová kerül a pénz és az ember, és ezzel alapvetően befolyásolja az egységek teljesítményét. Átcsoportosítással olyan megoldást találtál, amely az ügyfélnek jó. Csakhogy a terhet egy olyan csapatra tetted, amely nem kérte, és ez a két osztály viszonyát hosszú távon megmérgezheti.</t>
+          <t>Mintzberg erőforrás-elosztó szerepében a vezető dönti el, hová kerül a pénz és az ember, és ezzel alapvetően befolyásolja az egységek teljesítményét. Átcsoportosítással olyan megoldást találtál, amely az ügyfélnek jó. Csakhogy a terhet egy olyan csapatra raktad, amely nem kérte, és ez hosszú távon megmérgezheti a két osztály viszonyát.</t>
         </is>
       </c>
       <c r="H16" s="18" t="n">
@@ -3956,7 +3956,7 @@
       </c>
       <c r="E17" s="17" t="inlineStr">
         <is>
-          <t>Te húzod meg a határt: holnaptól nincs aznapi ígéret, kivétel nélkül. A hibák azonnal csökkennek, az értékesítők viszont a prémiumukat féltik.</t>
+          <t>Te húzod meg a határt: holnaptól nincs aznapi szállítás ígérete, kivétel nélkül. A hibák azonnal csökkennek, az értékesítők viszont a prémiumukat féltik.</t>
         </is>
       </c>
       <c r="F17" s="17" t="inlineStr">
@@ -3966,7 +3966,7 @@
       </c>
       <c r="G17" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg zavarelhárító szerepében a vezető gyorsan lép, amikor valami akadozik a működésben. A határozott szabály azonnal megállítja a hibák egyik forrását. Mivel viszont az érintettek nélkül született, az értékesítők a maguk módján fogják kerülgetni, és a prémiumuk kérdése megoldatlan marad.</t>
+          <t>Mintzberg zavarelhárító szerepében a vezető gyorsan lép, amikor valami akadozik a működésben. A határozott szabály azonnal megszünteti a hibák egyik forrását. Mivel azonban az érintettek nélkül született, az értékesítők a maguk módján meg fogják kerülni, és a prémiumuk kérdése sem oldódik meg.</t>
         </is>
       </c>
       <c r="H17" s="18" t="n">
@@ -3999,12 +3999,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>A havi jelentés</t>
+          <t>Az első havi jelentés</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Elkészül az első havi jelentés a patikaláncnak. Két mutató javult, egy — a panaszok lezárásának ideje — viszont romlott. Közben kapsz egy lelkes levelet egy szegedi patikustól, aki szerint soha nem volt ilyen jó a kiszolgálás. A jelentés holnap reggel megy ki.</t>
+          <t>Elkészül az első havi jelentés a patikalánc számára. Két mutató javult, egy viszont — a panaszok lezárásának ideje — romlott. Közben kapsz egy lelkes levelet egy szegedi patikustól, aki szerint még soha nem volt ilyen jó a kiszolgálás. A jelentésnek holnap reggel kell kimennie.</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Még egy hétig nem küldöd el, hátha addigra a harmadik mutató is javul. Tudod, hogy a patikalánc a pontos határidőket is figyeli.</t>
+          <t>Még egy hétig visszatartod, hátha addigra a harmadik mutató is javul. Tudod, hogy a patikalánc a határidők betartását is figyeli.</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>A jegyzet a döntés halogatásának nevezi, amikor menekülünk a probléma elől, és kivárjuk, hogy a helyzet magától rendeződjön. Egy hét múlva talán jobb számokat küldhetsz. Addig viszont épp azt a megbízhatóságot sérted, amelyért a patikalánc harcol: hogy időben kapja meg, amit ígértek neki.</t>
+          <t>A jegyzet a döntés halogatásának nevezi, amikor menekülünk a probléma elől, és kivárjuk, hogy a helyzet magától megoldódjon. Egy hét múlva talán jobb számokat küldhetsz. Addig viszont éppen azt a megbízhatóságot sérted, amelyért a patikalánc küzd: hogy időben megkapja, amit ígértek neki.</t>
         </is>
       </c>
       <c r="H18" s="12" t="n">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E19" s="17" t="inlineStr">
         <is>
-          <t>A számokat a tavaszi mélyponthoz hasonlítod, amikor minden mutató a legrosszabb volt. Így mindhárom javulásnak látszik, és semmi sem hamis benne.</t>
+          <t>A számokat a tavaszi mélyponthoz viszonyítod, amikor minden mutató a legrosszabb volt. Így mindhárom javulásnak látszik, és semmi sem hamis benne.</t>
         </is>
       </c>
       <c r="F19" s="17" t="inlineStr">
@@ -4072,7 +4072,7 @@
       </c>
       <c r="G19" s="17" t="inlineStr">
         <is>
-          <t>A kontraszt-hatás azt jelenti, hogy semmit nem ítélünk meg önmagában: mindig ahhoz mérjük, amivel előtte találkoztunk. Ha a tavaszi mélyponthoz viszonyítasz, minden javulásnak látszik. Egyik szám sem hamis, a kép mégis félrevezető, és ezt egy tapasztalt beszerzési vezető előbb-utóbb észre fogja venni.</t>
+          <t>A kontraszt-hatás azt jelenti, hogy semmit sem önmagában ítélünk meg, hanem mindig ahhoz mérjük, amivel előtte találkoztunk. Ha a tavaszi mélyponthoz viszonyítasz, minden javulásnak tűnik. Egyik szám sem hamis, a kép mégis félrevezető, és ezt egy tapasztalt beszerzési vezető előbb-utóbb észre fogja venni.</t>
         </is>
       </c>
       <c r="H19" s="18" t="n">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="E20" s="17" t="inlineStr">
         <is>
-          <t>A jelentés elejére a romló mutatót teszed, mellé pedig azt, mit csináltok vele. Tudod, hogy a patikalánc ettől idegesebb lesz, pont most, amikor kezd megnyugodni.</t>
+          <t>A jelentés elejére a romló mutatót teszed, és mellé azt, hogy mit tesztek ellene. Tudod, hogy ettől a patikalánc idegesebb lesz, éppen most, amikor kezdene megnyugodni.</t>
         </is>
       </c>
       <c r="F20" s="17" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G20" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg szóvivő szerepében a vezető a kívülállókat — ügyfeleket, partnereket — tájékoztatja a teljesítményről és a tervekről. Ha a rossz hírt te mondod el elsőként, megoldással együtt, a jó híreidnek is jobban hisznek majd. Most viszont egy olyan ügyfelet nyugtalanítasz, aki éppen kezdett megbékélni.</t>
+          <t>Mintzberg szóvivő szerepében a vezető a kívülállókat — ügyfeleket, partnereket — tájékoztatja a teljesítményről és a tervekről. Ha a rossz hírt te mondod el elsőként, a megoldással együtt, a jó híreidnek is jobban hisznek majd. Most viszont egy olyan ügyfelet nyugtalanítasz, aki éppen kezdett megbékélni.</t>
         </is>
       </c>
       <c r="H20" s="18" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="E21" s="17" t="inlineStr">
         <is>
-          <t>A jelentés elejére a szegedi patikus levelét teszed. Ez valódi visszajelzés, és jó hangulatot teremt a többi számhoz.</t>
+          <t>A jelentés elejére a szegedi patikus levelét teszed. Ez valódi visszajelzés, és jó hangulatot teremt a számokhoz.</t>
         </is>
       </c>
       <c r="F21" s="17" t="inlineStr">
@@ -4168,7 +4168,7 @@
       </c>
       <c r="G21" s="17" t="inlineStr">
         <is>
-          <t>A halo-effektus azt jelenti, hogy egyetlen kiemelkedő jellemző alapján alakul ki az általános benyomás. Egy lelkes levél az elején az egész jelentést jobb fénybe helyezi, még a romló mutatót is. A levél igaz, de nem reprezentatív, és ha az ügyfél később rájön, hogyan volt összerakva a jelentés, a következőnek már nem fog hinni.</t>
+          <t>A halo-effektus azt jelenti, hogy egyetlen kiemelkedő jellemző alapján alakul ki az általános benyomás. Egy lelkes levél az elején az egész jelentést jobb fénybe helyezi, még a romló mutatót is. A levél igaz, de nem reprezentatív, és ha az ügyfél később rájön, hogyan állt össze a jelentés, a következőnek már nem fog hinni.</t>
         </is>
       </c>
       <c r="H21" s="18" t="n">
@@ -4201,12 +4201,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Réka ötlete</t>
+          <t>Csevegőprogram vagy túlóra</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Réka új ötlettel jön: egy automatikus csevegőprogram, amely a patikák kérdéseinek negyven százalékára maga válaszolna. Az informatika szerint hat hét a bevezetés — a határidőig hét hét van hátra. A biztosabb, de drágább út a nyitvatartás meghosszabbítása túlórával. A pénz mindkettőre nem elég.</t>
+          <t>Réka új ötlettel áll elő: egy automatikus csevegőprogrammal, amely a patikák kérdéseinek negyven százalékára magától válaszolna. Az informatika szerint a bevezetés hat hétig tart, a határidőig pedig hét hét van hátra. A biztosabb, de drágább megoldás a nyitvatartás meghosszabbítása túlórával. A kettőre együtt nincs elég pénz.</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
@@ -4216,7 +4216,7 @@
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>Mindkettőt elindítod teljes erővel: a csevegőprogramot is, a túlórát is. A pénzt majd valahogy előteremted, a határidő fontosabb.</t>
+          <t>Mindkettőt teljes erővel elindítod: a csevegőprogramot is és a túlórát is. A pénzt majd valahogy előteremted, a határidő a fontosabb.</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
@@ -4226,7 +4226,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>James March hamisan pozitív hibának nevezi, amikor a döntéshozó olyan kontrollban hisz, amely a valóságban nincs meg. A „majd valahogy előteremtem” éppen ilyen hit. Rövid távon mindkét úton haladsz, de ha a pénz nem lesz meg, mindkettő félbemarad, és a csapat kétszer annyi munkával ér el feleannyit.</t>
+          <t>James March hamisan pozitív hibának nevezi, amikor a döntéshozó olyan kontrollban hisz, amely a valóságban nincs a kezében. A „majd valahogy előteremtem” éppen ilyen hit. Rövid távon mindkét úton haladsz, de ha nem lesz meg a pénz, mindkettő félbemarad, és a csapat kétszer annyi munkával feleannyit ér el.</t>
         </is>
       </c>
       <c r="H22" s="12" t="n">
@@ -4253,7 +4253,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="90" customHeight="1">
+    <row r="23" ht="76" customHeight="1">
       <c r="A23" s="15" t="n"/>
       <c r="B23" s="16" t="n"/>
       <c r="C23" s="17" t="n"/>
@@ -4264,7 +4264,7 @@
       </c>
       <c r="E23" s="17" t="inlineStr">
         <is>
-          <t>Rábólintasz Réka ötletére: ő ismeri a legjobban a patikák kérdéseit, és ő is fogja végigvinni. Te a háttérből támogatod.</t>
+          <t>Rábólintasz Réka ötletére: ő ismeri a legjobban a patikák kérdéseit, és ő is fogja végigvinni a projektet. Te a háttérből támogatod.</t>
         </is>
       </c>
       <c r="F23" s="17" t="inlineStr">
@@ -4274,7 +4274,7 @@
       </c>
       <c r="G23" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet csoportos döntési modelljei között szerepel a szakértői döntés: a csoport azt a tagját hagyja dönteni, aki a kérdésben a legjáratosabb. Réka tényleg ismeri a patikákat, és a bizalmad erőt ad neki. A modell hátránya, hogy nincs mellette ellenőrzés, és ha a program csúszik, egyetlen ember döntésén áll vagy bukik az egész.</t>
+          <t>A jegyzet csoportos döntési modelljei között szerepel a szakértői döntés: a csoport azt a tagját hagyja dönteni, aki az adott kérdésben a legjáratosabb. Réka valóban ismeri a patikákat, és a bizalmad erőt ad neki. A modell hátránya, hogy nincs mellette kontroll, és ha a program csúszik, minden egyetlen ember döntésén múlik.</t>
         </is>
       </c>
       <c r="H23" s="18" t="n">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="E24" s="17" t="inlineStr">
         <is>
-          <t>Leírsz három lehetőséget — a csevegőprogramot, a hosszabb nyitvatartást és a kettő kisebb változatát —, és mindegyiknél végiggondolod, mi történik, ha csúszik. Ez két nap, és Réka türelmetlen.</t>
+          <t>Leírsz három lehetőséget — a csevegőprogramot, a hosszabb nyitvatartást és a kettő kisebb léptékű kombinációját —, és mindegyiknél végiggondolod, mi történik, ha csúszik. Ez két napot vesz igénybe, és Réka türelmetlen.</t>
         </is>
       </c>
       <c r="F24" s="17" t="inlineStr">
@@ -4322,7 +4322,7 @@
       </c>
       <c r="G24" s="17" t="inlineStr">
         <is>
-          <t>Herbert Simon második döntési lépése a tervezés: a lehetséges cselekvési utak összegyűjtése és a várható következmények kiértékelése. Azzal, hogy a „mi van, ha csúszik” kérdést minden lehetőségnél feltetted, a kockázat láthatóvá vált. Két napot vesztesz, és Réka úgy érezheti, nem bízol benne.</t>
+          <t>Herbert Simon szerint a döntés második szakasza a tervezés: összegyűjtjük a lehetséges cselekvési utakat, és felmérjük a várható következményeiket. Azzal, hogy minden lehetőségnél feltetted a „mi lesz, ha csúszik?” kérdést, láthatóvá tetted a kockázatot. Két napot veszítesz, és Réka úgy érezheti, hogy nem bízol benne.</t>
         </is>
       </c>
       <c r="H24" s="18" t="n">
@@ -4349,7 +4349,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="76" customHeight="1">
+    <row r="25" ht="90" customHeight="1">
       <c r="A25" s="15" t="n"/>
       <c r="B25" s="16" t="n"/>
       <c r="C25" s="17" t="n"/>
@@ -4360,7 +4360,7 @@
       </c>
       <c r="E25" s="17" t="inlineStr">
         <is>
-          <t>A biztosat választod: hosszabb nyitvatartás, túlórával. Tudod, hogy ez működni fog, csak a csapat még jobban elfárad.</t>
+          <t>A biztos utat választod: hosszabb nyitvatartás, túlórával. Tudod, hogy ez működni fog, csak a csapat még jobban elfárad.</t>
         </is>
       </c>
       <c r="F25" s="17" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
-          <t>Simon szerint a valóságban nem az optimális, hanem az első elfogadható megoldást választjuk, mert az idő és az információ is korlátozott. A túlóra biztosan elég lesz a határidőig, és ez jogos szempont. A költséget viszont egy már kimerült csapat fizeti meg, és a határidő után semmi nem marad, ami tartósan javítaná a helyzetet.</t>
+          <t>Simon szerint a valóságban nem az optimális, hanem az első elfogadható megoldást választjuk, mert az időnk és az információnk is korlátozott. A túlóra a határidőig biztosan elég lesz, és ez jogos szempont. Az árát viszont egy már most is kimerült csapat fizeti meg, és a határidő után semmi sem marad, ami tartósan javítana a helyzeten.</t>
         </is>
       </c>
       <c r="H25" s="18" t="n">
@@ -4403,12 +4403,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Tízből egy rossz válasz</t>
+          <t>A hibázó csevegőprogram</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>A hatodik héten a csevegőprogram elkészül. A tesztek szerint minden tizedik kérdésre rossz választ ad — például téves nyitvatartást mond egy patikáról. Ha most nem indul el, a határidőig már nem fog. A szerverteremben az informatikusok rád néznek.</t>
+          <t>A hatodik héten elkészül a csevegőprogram. A tesztek szerint minden tizedik kérdésre rossz választ ad: például téves nyitvatartást mond egy patikáról. Ha most nem indul el, a határidőig már nem fog. A szerverteremben az informatikusok rád néznek.</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
@@ -4418,7 +4418,7 @@
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>Nem indítjátok el, amíg a hibaarány egy százalék alá nem megy. Egy rossz nyitvatartási adat egy betegnek komoly gondot okozhat, még ha így lekésitek is a határidőt.</t>
+          <t>Addig nem indítjátok el, amíg a hibaarány egy százalék alá nem csökken. Egy rossz nyitvatartási adat komoly gondot okozhat egy betegnek, még ha így le is késitek a határidőt.</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Simon szerint a jól strukturált döntésnél világos, mi a probléma, a rosszul strukturáltnál viszont ez sem egyértelmű. Egy egyszázalékos küszöbbel jól strukturált, műszaki kérdéssé alakítottad az indítást. Csakhogy a valódi kérdés az, mit tart fontosabbnak az ügyfél: a pontos határidőt vagy a hibátlanságot — és ezt nem kérdezted meg tőle.</t>
+          <t>Simon szerint a jól strukturált döntésnél világos, mi a probléma, a rosszul strukturáltnál viszont még ez sem egyértelmű. Az egyszázalékos küszöbbel jól strukturált, műszaki kérdéssé alakítottad az indítást. Csakhogy a valódi kérdés az, hogy az ügyfélnek mi a fontosabb: a határidő vagy a hibátlanság — és ezt nem kérdezted meg tőle.</t>
         </is>
       </c>
       <c r="H26" s="12" t="n">
@@ -4466,7 +4466,7 @@
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>Csak tíz patikában indítjátok el, próbaképp. A patikalánc egésze így nem látja az eredményt a határidőre, de a hibák kis körben maradnak.</t>
+          <t>Próbaképpen csak tíz patikában indítjátok el. A patikalánc egésze így nem látja az eredményt a határidőre, a hibák viszont szűk körben maradnak.</t>
         </is>
       </c>
       <c r="F27" s="17" t="inlineStr">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="G27" s="17" t="inlineStr">
         <is>
-          <t>Az inkrementalizmus a nagy, egyszeri lépések helyett kis, fokozatos korrekciókat jelent, amelyekből menet közben tanulni lehet. A próbaüzem kicsiben mutatja meg, mi működik és mi nem. A határidőre viszont nem lesz látványos eredmény, és a patikalánc ezt könnyen óvatoskodásnak láthatja.</t>
+          <t>Az inkrementalizmus azt jelenti, hogy nagy, egyszeri lépések helyett kis, fokozatos korrekciókkal haladunk, és menet közben tanulunk. A próbaüzem kicsiben megmutatja, mi működik és mi nem. A határidőre viszont nem lesz látványos eredmény, és a patikalánc ezt könnyen óvatoskodásnak láthatja.</t>
         </is>
       </c>
       <c r="H27" s="18" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="E28" s="17" t="inlineStr">
         <is>
-          <t>Mindenhol elindítjátok, a hibákat menet közben javítjátok. A határidő tartható, és a patikalánc végre valami nagyot lát.</t>
+          <t>Mindenhol elindítjátok, a hibákat pedig menet közben javítjátok. A határidő tartható, és a patikalánc végre valami nagyot lát.</t>
         </is>
       </c>
       <c r="F28" s="17" t="inlineStr">
@@ -4524,7 +4524,7 @@
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
-          <t>A diszkontálás az a hajlamunk, hogy a közeli dolgokat felértékeljük, a távolabbiakat leértékeljük. A határidő itt van előtted, a rossz válaszok okozta bosszúság viszont csak később, szétszórva jelentkezik. A határidőt tartod, de ha a hibák összeadódnak, éppen a megbízhatóságot sérted, amiért az egész munka indult.</t>
+          <t>A diszkontálás az a hajlamunk, hogy a közeli dolgokat túlértékeljük, a távolabbiakat pedig alábecsüljük. A határidő itt van előtted, a rossz válaszok okozta bosszúság viszont csak később és szétszórva jelentkezik. A határidőt tartod, de ha a hibák összeadódnak, éppen azt a megbízhatóságot sérted, amiért az egész munka elindult.</t>
         </is>
       </c>
       <c r="H28" s="18" t="n">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="E29" s="17" t="inlineStr">
         <is>
-          <t>Elindítjátok, de minden válasz alatt ott a gomb: „Kérem, hívjon vissza egy munkatárs.” Így a hibás válaszok egy része is ember elé kerül, csak kicsit később.</t>
+          <t>Elindítjátok, de minden válasz alatt ott lesz egy gomb: „Kérem, hívjon vissza egy munkatárs.” Így a hibás válaszok egy része is emberhez kerül, csak kicsit később.</t>
         </is>
       </c>
       <c r="F29" s="17" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="G29" s="17" t="inlineStr">
         <is>
-          <t>Snowden és Boone szerint komplex helyzetben nincs előre biztos válasz: olyan lépéseket kell tenni, amelyekből tanulni lehet, és amelyek kudarca nem végzetes. A visszahívás gomb ilyen biztonsági háló: a program élesben tanul, a hibáit pedig ember fogja meg. Ennek ára, hogy néhány rossz válasz így is eljut a patikákhoz, és a csapatra plusz munka hárul.</t>
+          <t>Snowden és Boone szerint komplex helyzetben nincs előre biztos válasz: olyan lépéseket kell tenni, amelyekből tanulni lehet, és amelyek kudarca nem végzetes. A visszahívás gomb ilyen biztonsági háló: a program éles használat közben tanul, a hibáit pedig ember szűri ki. Ennek ára, hogy néhány rossz válasz így is eljut a patikákhoz, és a csapatra többletmunka hárul.</t>
         </is>
       </c>
       <c r="H29" s="18" t="n">
@@ -4605,12 +4605,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Három ajánlat</t>
+          <t>Szerződési ajánlatok mérlegelése</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>A tizedik héten a patikalánc visszaír: maradnának, de két lehetőséget kínálnak — hároméves szerződés tizenöt százalék árengedménnyel, vagy egyéves szerződés a mostani áron, szigorú kötbérrel. Gábor közben két kisebb ügyfelet is felhozott, akik együtt pótolhatnák a patikaláncot, ha elengednétek. Holnapig kell válaszolni. A tárgyalóban ott ül veled a pénzügyi igazgató és Gábor.</t>
+          <t>A tizedik héten a patikalánc válaszol: maradnának, és két lehetőséget kínálnak. Az egyik egy hároméves szerződés tizenöt százalékos árengedménnyel, a másik egy egyéves szerződés a mostani áron, de szigorú kötbérrel. Gábor közben két kisebb ügyfelet is hozott, akik együtt pótolhatnák a patikaláncot, ha elengednétek. Holnapig kell válaszolni. A tárgyalóban ott ül veled a pénzügyi igazgató és Gábor.</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
@@ -4620,7 +4620,7 @@
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>Holnap reggel a csapatodat is megkérdezed: nekik kell majd teljesíteniük, akármelyik mellett döntötök. Tudod, hogy a hír így kiszivároghat a tárgyalás előtt.</t>
+          <t>Holnap reggel a csapatodat is megkérdezed, hiszen nekik kell majd teljesíteniük, akármelyik mellett döntötök. Tudod, hogy így a hír a tárgyalás előtt kiszivároghat.</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>A jegyzet csoportos döntési modelljei közül a konzultatív döntésnél a vezető meghallgatja a csoport véleményét, de a döntést ő hozza meg. A csapat tudja, mit bír el, és ha megkérdezed, a végrehajtásban is jobban kitart melletted. Az ára az idő, és az, hogy egy érzékeny tárgyalási pozíció több ember kezébe kerül.</t>
+          <t>A jegyzet csoportos döntési modelljei közül a konzultatív döntésnél a vezető meghallgatja a csoport véleményét, de a döntést ő maga hozza meg. A csapat tudja, mennyit bír el, és ha megkérdezed, a végrehajtás során is jobban kitart melletted. Az ára az idő, és az, hogy egy érzékeny tárgyalási pozíció több ember kezébe kerül.</t>
         </is>
       </c>
       <c r="H30" s="12" t="n">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="E31" s="17" t="inlineStr">
         <is>
-          <t>A hároméves szerződést választod: az elmúlt hónapok után a biztonság a legfontosabb, még ha kevesebb is a haszon.</t>
+          <t>A hároméves szerződést választod: az elmúlt hónapok után a biztonság a legfontosabb, még ha kisebb is a haszon.</t>
         </is>
       </c>
       <c r="F31" s="17" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="G31" s="17" t="inlineStr">
         <is>
-          <t>Az utólagossági hatás azt jelenti, hogy a legfrissebb, legélénkebb élmény köré szervezzük a megítélést. A majdnem elveszített ügyfél emléke olyan erős, hogy minden mást a biztonság mögé soroltál. Ez érthető és védhető, de három évre olcsóbban kötöd le a cég legnagyobb bevételét, és a csapatnak ugyanazt kell nyújtania kevesebb pénzért.</t>
+          <t>Az utólagossági hatás azt jelenti, hogy a legfrissebb, legélénkebb élmény köré rendezzük a megítélést. A majdnem elveszített ügyfél emléke olyan erős, hogy minden mást a biztonság mögé soroltál. Ez érthető és védhető, de három évre olcsóbban kötöd le a cég legnagyobb bevételét, és a csapatnak ugyanazt kell teljesítenie kevesebb pénzért.</t>
         </is>
       </c>
       <c r="H31" s="18" t="n">
@@ -4716,7 +4716,7 @@
       </c>
       <c r="E32" s="17" t="inlineStr">
         <is>
-          <t>Egymás mellé teszitek a három lehetőséget bevétel, kockázat, a csapat terhelése és a hosszú távú kapcsolat szerint, és először megnézitek, van-e olyan, amelyik mindenben rosszabb valamelyik másiknál. Ez éjfélig tart.</t>
+          <t>Egymás mellé teszitek a három lehetőséget a bevétel, a kockázat, a csapat terhelése és a hosszú távú kapcsolat szerint, és először megnézitek, van-e köztük olyan, amelyik mindenben rosszabb valamelyik másiknál. Ez éjfélig eltart.</t>
         </is>
       </c>
       <c r="F32" s="17" t="inlineStr">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="G32" s="17" t="inlineStr">
         <is>
-          <t>A dominancia elve szerint ha egy lehetőség semmiben nem jobb egy másiknál, és legalább egy szempontból rosszabb, kihúzhatjuk, mielőtt a nehéz mérlegelésbe kezdenénk. Ez leszűkíti a döntést a valódi versenyzőkre. Maga a választás — mennyi kockázatot ér meg a nagyobb haszon — így is a tiéd marad, és az éjszaka is rámegy.</t>
+          <t>A dominancia elve szerint ha egy lehetőség semmiben sem jobb egy másiknál, és legalább egy szempontból rosszabb, kihúzhatjuk, mielőtt a nehéz mérlegelésbe kezdenénk. Így a döntés a valódi esélyesekre szűkül. Maga a választás — mennyi kockázatot ér meg a nagyobb haszon — ettől még a te dolgod marad, és az éjszaka is rámegy.</t>
         </is>
       </c>
       <c r="H32" s="18" t="n">
@@ -4774,7 +4774,7 @@
       </c>
       <c r="G33" s="17" t="inlineStr">
         <is>
-          <t>Az ezredes-hatás az a hajlamunk, hogy a magas beosztású vagy nagy tekintélyű emberek szavát hitelesebbnek tartjuk. A pénzügyi igazgató tényleg jól látja a számokat, de a csapat terhelését és az ügyfélkapcsolatot nem ő ismeri a legjobban. A döntés szakszerű lesz, a felelősség viszont kicsúszik a kezedből.</t>
+          <t>Az ezredes-hatás az a hajlamunk, hogy a magas beosztású vagy nagy tekintélyű emberek szavát hitelesebbnek tartjuk. A pénzügyi igazgató valóban jól látja a számokat, de a csapat terhelését és az ügyfélkapcsolatot nem ő ismeri a legjobban. A döntés szakszerű lesz, a felelősség viszont kicsúszik a kezedből.</t>
         </is>
       </c>
       <c r="H33" s="18" t="n">
@@ -4807,12 +4807,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Negyed tizenkettő</t>
+          <t>Adatszivárgás az aláírás előtt</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Az aláírás előtti éjjel negyed tizenkettőkor felhív az ügyeletes informatikus. A csevegőprogram egy beállítási hiba miatt három órán át mások számára is láthatóvá tette kétezer patikai vásárló adatait, köztük gyógyszerneveket. A hibát már kijavították, kívülről senki nem tud róla. Az aláírás reggel tízkor lesz, és a cég bevételének negyede múlik rajta.</t>
+          <t>Az aláírás előtti éjjel negyed tizenkettőkor felhív az ügyeletes informatikus. A csevegőprogram egy beállítási hiba miatt három órán át mások számára is láthatóvá tette kétezer patikai vásárló adatait, köztük gyógyszerneveket is. A hibát már kijavították, és kívülről senki sem tud róla. Az aláírás reggel tízkor lesz, és a cég bevételének negyede múlik rajta.</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>Még éjjel felhívod a vezérigazgatót, reggel pedig — az aláírás előtt — elmondjátok a patikaláncnak. Tudod, hogy ezzel a szerződés is elveszhet.</t>
+          <t>Még éjjel felhívod a vezérigazgatót, reggel pedig — még az aláírás előtt — elmondjátok a patikaláncnak. Tudod, hogy így a szerződés is elveszhet.</t>
         </is>
       </c>
       <c r="F34" s="11" t="inlineStr">
@@ -4832,7 +4832,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>A napfény teszt egyetlen kérdés: jól érezném magam, ha ez a döntés minden részletével együtt nyilvánosságra kerülne? Ha az ügyfél utólag tudja meg, hogy az aláíráskor már ismerted a hibát, azt nem fogod tudni megmagyarázni. Az őszinteség ára lehet a szerződés — és vele az állások egy része.</t>
+          <t>A napfény teszt egyetlen kérdés: jól érezném-e magam, ha ez a döntés minden részletével együtt nyilvánosságra kerülne? Ha az ügyfél utólag tudja meg, hogy az aláíráskor már ismerted a hibát, azt nem fogod tudni megmagyarázni. Az őszinteség ára lehet a szerződés — és vele együtt az állások egy része.</t>
         </is>
       </c>
       <c r="H34" s="12" t="n">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="E35" s="17" t="inlineStr">
         <is>
-          <t>Reggelig nem szólsz senkinek: egyedül, az informatikussal kivizsgáljátok, pontosan kiket érintett a hiba, és csak utána döntesz a bejelentésről.</t>
+          <t>Reggelig senkinek sem szólsz: az informatikussal kettesben kivizsgáljátok, pontosan kiket érintett a hiba, és csak utána döntesz a bejelentésről.</t>
         </is>
       </c>
       <c r="F35" s="17" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="G35" s="17" t="inlineStr">
         <is>
-          <t>Az autokratikus döntésnél a vezető egyedül dönt, mások minimális közreműködésével. A jegyzet szerint ez válsághelyzetben, időhiányban indokolt lehet, és most valóban nincs idő hosszú egyeztetésre. A kockázat az, hogy egyedül viszel egy olyan terhet, amelyről a vezérigazgatónak is tudnia kellene, és reggelre már csak kevés lehetőség marad.</t>
+          <t>Az autokratikus döntésnél a vezető egyedül dönt, mások alig vesznek részt benne. A jegyzet szerint ez válsághelyzetben, időhiány esetén indokolt lehet, és most valóban nincs idő hosszas egyeztetésre. A kockázat az, hogy egyedül cipelsz egy olyan terhet, amelyről a vezérigazgatónak is tudnia kellene, és reggelre már alig marad mozgástered.</t>
         </is>
       </c>
       <c r="H35" s="18" t="n">
@@ -4918,7 +4918,7 @@
       </c>
       <c r="E36" s="17" t="inlineStr">
         <is>
-          <t>Még éjjel felhívod a patikalánc vezetőjét, négyszemközt elmondod, mi történt, és megkérdezed, hogyan kezeljétek közösen. Ezzel őt is nehéz helyzetbe hozod.</t>
+          <t>Még éjjel felhívod a patikalánc vezetőjét, négyszemközt elmondod neki, mi történt, és megkérdezed, hogyan kezeljétek közösen. Ezzel őt is nehéz helyzetbe hozod.</t>
         </is>
       </c>
       <c r="F36" s="17" t="inlineStr">
@@ -4928,7 +4928,7 @@
       </c>
       <c r="G36" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg tárgyaló szerepében a vezető a másik féllel közösen alakítja ki a megoldást. Az ügyfél így nem utólag, hanem időben tudja meg a hibát, és beleszólhat a kezelésébe. Csakhogy a kényes döntés egy részét rá terhelted, és a saját céged vezetése kimaradt a legfontosabb beszélgetésből.</t>
+          <t>Mintzberg tárgyaló szerepében a vezető a másik féllel közösen alakítja ki a megoldást. Így az ügyfél nem utólag, hanem időben értesül a hibáról, és beleszólhat a kezelésébe. Csakhogy a kényes döntés egy részét ráterhelted, a saját céged vezetése pedig kimaradt a legfontosabb beszélgetésből.</t>
         </is>
       </c>
       <c r="H36" s="18" t="n">
@@ -4966,7 +4966,7 @@
       </c>
       <c r="E37" s="17" t="inlineStr">
         <is>
-          <t>Aláírtok, és utána, a törvényes határidőn belül jelentitek az incidenst. Nem hazudsz, csak a sorrendet választod meg úgy, hogy háromszáz ember állása ne kerüljön veszélybe.</t>
+          <t>Aláírtok, és utána, a törvényes határidőn belül jelentitek az incidenst. Nem hazudsz, csak úgy választod meg a sorrendet, hogy háromszáz ember állása ne kerüljön veszélybe.</t>
         </is>
       </c>
       <c r="F37" s="17" t="inlineStr">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="G37" s="17" t="inlineStr">
         <is>
-          <t>A gátló racionalizálások olyan érvek, amelyekkel egy kétes döntést magunk előtt elfogadhatóvá teszünk. A „jó célt szolgál” itt valódi célt véd: háromszáz ember állását. A hozzá vezető út mégis az, hogy az ügyfél egy számára fontos tény ismerete nélkül írja alá a szerződést — és ezt később nem lehet visszacsinálni.</t>
+          <t>A gátló racionalizálások olyan érvek, amelyekkel egy kétes döntést a saját szemünkben elfogadhatóvá teszünk. A „jó célt szolgál” itt valódi célt véd: háromszáz ember állását. A hozzá vezető út azonban az, hogy az ügyfél egy számára fontos tény ismerete nélkül írja alá a szerződést — és ezt később nem lehet visszacsinálni.</t>
         </is>
       </c>
       <c r="H37" s="18" t="n">
@@ -5003,18 +5003,18 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="76" customHeight="1">
+    <row r="38" ht="90" customHeight="1">
       <c r="A38" s="9" t="n">
         <v>10</v>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Hétfő reggel</t>
+          <t>Visszatekintés a csapattal</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>A három hónap véget ért. Hétfő reggel a csapat összegyűlik a csapatszobában. Voltak, akik hatvanórás heteket húztak le. A vezérigazgató kért egy diát arról, mit tanult a cég, a csapat pedig azt kérdezi tőled: mi lesz velünk ezután?</t>
+          <t>A három hónap véget ért. Hétfő reggel a csapat összegyűlik a csapatszobában. Volt, aki hatvanórás heteket dolgozott végig. A vezérigazgató kért egy diát arról, mit tanult a cég ebből az időszakból, a csapat pedig azt kérdezi tőled: mi lesz velünk ezután?</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>Elmondod, hol hibáztál te, mit gondoltál rosszul az elején, és megkérdezed őket, ők mit csinálnának másképp. A diára is ez kerül.</t>
+          <t>Elmondod, hol hibáztál, mit gondoltál rosszul az elején, és megkérdezed őket, ők mit csinálnának másképp. A diára is ez kerül.</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>A következtetési létra azt mutatja be, milyen gyorsan jutunk a látott tényekből feltevésekhez és ítéletekhez; a reflektív gondolkodás ezen a létrán való tudatos lemászás. Ha kimondod, melyik feltevésed volt téves, a csapat is mer majd ugyanígy gondolkodni. A vezérigazgató szemében viszont ez a dia kevésbé lesz fényes.</t>
+          <t>A következtetési létra azt mutatja be, milyen gyorsan jutunk el a látott tényektől a feltevésekig és az ítéletekig; a reflektív gondolkodás azt jelenti, hogy tudatosan visszamászunk ezen a létrán. Ha kimondod, melyik feltevésed volt téves, a csapat is mer majd így gondolkodni. A vezérigazgató szemében viszont ez a dia kevésbé lesz fényes.</t>
         </is>
       </c>
       <c r="H38" s="12" t="n">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="E39" s="17" t="inlineStr">
         <is>
-          <t>Megköszönöd a munkájukat, és bejelented a következő nagy célt. Úgy gondolod, most a lendületre van szükség, nem a múlt boncolgatására.</t>
+          <t>Megköszönöd a munkájukat, és bejelented a következő nagy célt. Úgy gondolod, most lendületre van szükség, nem a múlt boncolgatására.</t>
         </is>
       </c>
       <c r="F39" s="17" t="inlineStr">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="G39" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet háromféle vezetői stratégiát különít el: a problémakeresőt, a problémamegoldót és a problémakerülőt, aki a nehéz kérdéseket inkább figyelmen kívül hagyja. A lendület valóban fontos, és a köszönet is jár. Ha viszont a három hónap tanulságai kimaradnak, a következő válságban ugyanazokat a hibákat fogjátok elkövetni.</t>
+          <t>A jegyzet háromféle vezetői stratégiát különít el: a problémakeresőt, a problémamegoldót és a problémakerülőt, aki a nehéz kérdésekről inkább nem vesz tudomást. A lendület valóban fontos, és a köszönet is jár. Ha viszont a három hónap tanulságai kimaradnak, a következő válságban ugyanazokat a hibákat fogjátok elkövetni.</t>
         </is>
       </c>
       <c r="H39" s="18" t="n">
@@ -5120,7 +5120,7 @@
       </c>
       <c r="E40" s="17" t="inlineStr">
         <is>
-          <t>A vezérigazgatónak szánt diára a sikerek a csapat érdemeként, a gondok a nehéz körülmények — a túlterhelés, a határidő — következményeként kerülnek. A csapat büszke lehet magára.</t>
+          <t>A vezérigazgatónak szánt diára a sikereket a csapat érdemeként, a gondokat pedig a nehéz körülmények — a túlterhelés és a határidő — következményeként írod fel. A csapat büszke lehet magára.</t>
         </is>
       </c>
       <c r="F40" s="17" t="inlineStr">
@@ -5130,7 +5130,7 @@
       </c>
       <c r="G40" s="17" t="inlineStr">
         <is>
-          <t>Az énmegerősítő attribúció az a hajlamunk, hogy a sikereket magunknak, a kudarcokat a körülményeknek tulajdonítsuk; ez egy csapattal együtt is működik. A dia büszkeséget ad, és a körülmények valóban nehezek voltak. Így viszont senki nem néz szembe azzal, mit lehetett volna jobban csinálni, és a vezérigazgató sem kap valódi tanulságot.</t>
+          <t>Az énmegerősítő attribúció az a hajlamunk, hogy a sikereket magunknak, a kudarcokat pedig a körülményeknek tulajdonítjuk; ez egy egész csapatra is igaz lehet. A dia büszkeséget ad, és a körülmények valóban nehezek voltak. Így viszont senki sem néz szembe azzal, mit lehetett volna jobban csinálni, és a vezérigazgató sem kap valódi tanulságot.</t>
         </is>
       </c>
       <c r="H40" s="18" t="n">
@@ -5178,7 +5178,7 @@
       </c>
       <c r="G41" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg információgyűjtő szerepében a vezető a szervezet belső információáramlásának központja. A névtelenség miatt olyan dolgok is felszínre kerülnek, amelyeket szemtől szemben senki nem mondana ki. A szűrés viszont nálad marad, és a csapat nem látja, mi lett a véleményéből.</t>
+          <t>Mintzberg információgyűjtő szerepében a vezető a szervezeten belüli információáramlás központja. A névtelenségnek köszönhetően olyan dolgok is felszínre kerülnek, amelyeket szemtől szemben senki sem mondana ki. A szűrés viszont a te kezedben marad, és a csapat nem látja, mi lett a véleményéből.</t>
         </is>
       </c>
       <c r="H41" s="18" t="n">
@@ -5360,18 +5360,18 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="76" customHeight="1">
+    <row r="2" ht="90" customHeight="1">
       <c r="A2" s="9" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>Négy óra</t>
+          <t>Éjszakai riasztás</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Éjjel egykor riasztás: az ezrednek négy órán belül el kell indulnia Tiszaszögre, ahol hat nap múlva tetőzik az árhullám. Az állomány fele hétvégi eltávozáson van, a laktanya kapujánál a teherautók már járatják a motort. A parancs szerint indulni kell — a kérdés az, hogyan.</t>
+          <t>Éjjel egykor riasztás: az ezrednek négy órán belül el kell indulnia Tiszaszögre, ahol hat nap múlva tetőzik az árhullám. Az állomány fele hétvégi eltávozáson van, a laktanya kapujánál már indulásra készen állnak a teherautók. A parancs szerint mindenkinek indulnia kell — a kérdés csak az, hogyan.</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
@@ -5381,7 +5381,7 @@
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>Előreküldesz egy tízfős felderítő csapatot egy mérnökkel, te pedig négy óra múlva jössz a többiekkel. Mire megérkezel, már tudod, mi vár rátok.</t>
+          <t>Előreküldesz egy tízfős felderítőcsoportot egy mérnökkel, te pedig négy óra múlva követed őket a többiekkel. Mire megérkezel, már tudod, mi vár rátok.</t>
         </is>
       </c>
       <c r="F2" s="11" t="inlineStr">
@@ -5391,7 +5391,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Herbert Simon szerint a döntés első lépése a megértés: a helyzetről szóló tudás összegyűjtése, még a tervezés előtt. A felderítők miatt nem vakon érkezel, és az első óráid terve a valóságra épül. Cserébe eltértél a parancstól, amely az ezred együttes indulásáról szólt, és a kis csapat egy darabig magára marad.</t>
+          <t>Herbert Simon szerint a döntés első szakasza a megértés: összegyűjtjük a helyzetről szóló tudást, még mielőtt tervezni kezdenénk. A felderítőknek köszönhetően nem vakon érkezel, és az első óráid terve a valóságra épül. Cserébe eltértél a parancstól, amely az ezred együttes indulásáról szólt, és a kis csoport egy ideig magára marad.</t>
         </is>
       </c>
       <c r="H2" s="12" t="n">
@@ -5429,7 +5429,7 @@
       </c>
       <c r="E3" s="17" t="inlineStr">
         <is>
-          <t>Felhívod az elöljárót, és kéred, hogy tolják ki az indulást, amíg összeszeded az embereket. Így rendezetten mehettek, de órákat veszítetek.</t>
+          <t>Felhívod az elöljáródat, és kéred, hogy halasszák el az indulást, amíg összeszeded az embereket. Így rendezetten indulhattok, de órákat veszítetek.</t>
         </is>
       </c>
       <c r="F3" s="17" t="inlineStr">
@@ -5439,7 +5439,7 @@
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet a döntés halogatásának nevezi, amikor a problémát tovább toljuk, és kivárjuk, amíg a helyzet kikényszeríti a lépést. Őszintén jelezted a gondot, és az embereidre is gondoltál. A víz viszont nem vár, és az elöljáró azt látja, hogy az első órában egy parancs megváltoztatásán dolgozol, nem a végrehajtásán.</t>
+          <t>A jegyzet a döntés halogatásának nevezi, amikor a problémát magunk előtt görgetjük, és kivárjuk, amíg a helyzet kikényszeríti a lépést. Őszintén jelezted a gondot, és az embereidre is gondoltál. A víz viszont nem vár, az elöljáród pedig azt látja, hogy az első órában a parancs megváltoztatásán dolgozol, nem a végrehajtásán.</t>
         </is>
       </c>
       <c r="H3" s="18" t="n">
@@ -5477,7 +5477,7 @@
       </c>
       <c r="E4" s="17" t="inlineStr">
         <is>
-          <t>A jelenlévőkkel négy órán belül elindulsz, a többieket egyenesen a helyszínre rendeled. Az első két napban fél létszámmal dolgoztok, de ott vagytok.</t>
+          <t>A jelen lévőkkel négy órán belül elindulsz, a többieket pedig egyenesen a helyszínre rendeled. Az első két napban fél létszámmal dolgoztok, de ott vagytok.</t>
         </is>
       </c>
       <c r="F4" s="17" t="inlineStr">
@@ -5487,7 +5487,7 @@
       </c>
       <c r="G4" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg zavarelhárító szerepében a vezető gyorsan lép, amikor valami megzavarja a működést. Időben a helyszínen lenni itt valódi érték, és a parancsot is betartottad. Az ár az, hogy fél létszámmal a jelenlévők az első napokban túlterhelődnek, és a kimerültség később visszaüthet.</t>
+          <t>Mintzberg zavarelhárító szerepében a vezető gyorsan lép, amikor valami megzavarja a működést. Itt valódi érték, hogy időben a helyszínen vagytok, és a parancsot is betartottad. Az ára, hogy az első napokban a fél létszám túlterhelődik, és a kimerültség később visszaüthet.</t>
         </is>
       </c>
       <c r="H4" s="18" t="n">
@@ -5514,7 +5514,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="62" customHeight="1">
+    <row r="5" ht="76" customHeight="1">
       <c r="A5" s="15" t="n"/>
       <c r="B5" s="16" t="n"/>
       <c r="C5" s="17" t="n"/>
@@ -5525,7 +5525,7 @@
       </c>
       <c r="E5" s="17" t="inlineStr">
         <is>
-          <t>Visszarendelsz mindenkit, és csak teljes létszámmal indultok, nyolc óra múlva. A szabályzat szerint így kell kivonulni, és így senki nem marad magára.</t>
+          <t>Visszarendelsz mindenkit, és csak teljes létszámmal indultok, nyolc óra múlva. A szabályzat szerint így kell kivonulni, és így senki sem kap kivételes elbánást.</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
-          <t>Simon programozott döntésnek nevezi azt, amelyre kész rutin vagy szabály van. A kivonulási rend ilyen rutin, és sok helyzetben éppen ez ad biztonságot. Egy rendkívüli árhullámnál viszont a szabály szerinti nyolc óra olyan idő, amely a helyszínen hiányozni fog.</t>
+          <t>Simon programozott döntésnek nevezi azt, amelyre kész rutin vagy szabály létezik. A kivonulási rend ilyen rutin, és sok helyzetben éppen ez ad biztonságot. Egy rendkívüli árhullámnál viszont a szabály szerinti nyolc órával olyan időt veszítesz, amely a helyszínen hiányozni fog.</t>
         </is>
       </c>
       <c r="H5" s="18" t="n">
@@ -5568,12 +5568,12 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Kinek a gátja?</t>
+          <t>Az erők elosztása</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Megérkeztetek. A törzssátorban a térkép fölé hajol Kiss polgármester, Varga, a vízügyi mérnök és a gazdák képviselője. Varga szerint minden erőt a városi gátra kell összpontosítani. A gazdák szerint ha a tanyák feletti töltés átszakad, elvész a termés és negyven család megélhetése. Mindenki tőled várja, hová küldöd az embereket.</t>
+          <t>Megérkeztetek. A törzssátorban a térkép fölé hajol Kiss polgármester, Varga, a vízügyi mérnök és a gazdák képviselője. Varga szerint minden erőt a városi gátra kell összpontosítani. A gazdák szerint viszont ha a tanyák feletti töltés átszakad, odavész a termés és negyven család megélhetése. Mindenki tőled várja, hová küldöd az embereket.</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Fele-fele arányban osztod el az erőket a városi és a tanyasi töltés között, hogy senki ne mondhassa, hogy cserben hagytad.</t>
+          <t>Fele-fele arányban osztod el az erőket a városi és a tanyasi töltés között, hogy senki se mondhassa, hogy cserben hagytad.</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
@@ -5593,7 +5593,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Simon szerint a valóságban nem az optimális, hanem az első elfogadható megoldást szoktuk választani. A fele-fele elosztás mindenkinek elfogadható, és a vitát azonnal lezárja. Csakhogy a víz nem egyenlően fenyeget, és ha egyik helyen sem lesz elég ember, mindkét töltés gyengébb marad a kelleténél.</t>
+          <t>Simon szerint a valóságban nem az optimális, hanem az első elfogadható megoldást szoktuk választani. A fele-fele elosztás mindenkinek elfogadható, és azonnal lezárja a vitát. Csakhogy a víz nem egyformán fenyeget, és ha egyik helyen sem lesz elég ember, mindkét töltés gyengébb marad a kelleténél.</t>
         </is>
       </c>
       <c r="H6" s="12" t="n">
@@ -5620,7 +5620,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="76" customHeight="1">
+    <row r="7" ht="90" customHeight="1">
       <c r="A7" s="15" t="n"/>
       <c r="B7" s="16" t="n"/>
       <c r="C7" s="17" t="n"/>
@@ -5641,7 +5641,7 @@
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet a döntéshozói magatartások között írja le a döntés elhárítását, amikor a vezető másra hagyja, amit neki kellene eldöntenie. A polgármester valóban ismeri a várost, és a helyiek jobban elfogadják a szavát. De az ezred a te felelősséged, és ha rosszul alakul, senki nem fogja a polgármestert kérdezni.</t>
+          <t>A jegyzet a döntéshozói magatartások között írja le a döntés elhárítását: a vezető másra hagyja azt, amit neki kellene eldöntenie. A polgármester valóban ismeri a várost, és a helyiek is jobban elfogadják a szavát. Az ezred azonban a te felelősséged, és ha rosszul alakulnak a dolgok, senki sem a polgármestert fogja kérdőre vonni.</t>
         </is>
       </c>
       <c r="H7" s="18" t="n">
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E8" s="17" t="inlineStr">
         <is>
-          <t>Mielőtt bárhová küldesz valakit, felírjátok, kik mind érintettek — városiak, tanyasiak, gazdák, a kórház, a katonák —, kinek mi forog kockán, és kinek mekkora a beleszólása. Ez egy óra, amíg a víz emelkedik.</t>
+          <t>Mielőtt bárkit bárhová küldenél, végiggondoljátok, kik az érintettek, kinek mi forog kockán, és kinek mekkora a beleszólása. Ez egy óra, miközben a víz emelkedik.</t>
         </is>
       </c>
       <c r="F8" s="17" t="inlineStr">
@@ -5689,7 +5689,7 @@
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>Az érintett-térkép megmutatja, kikre hat egy döntés, azokat is beleértve, akik nem ülnek az asztalnál — itt például a kórházat vagy a tanyán élő időseket. Ettől lesz látható, kinek a hangja hiányzik a sátorból. Egy óra ilyenkor sok, és a sátor előtt várakozó katonák nem értik, miért nem indulnak még.</t>
+          <t>Az érintett-térkép megmutatja, kikre hat egy döntés, azokat is beleértve, akik nem ülnek az asztalnál — itt például a kórházat vagy a tanyákon élő időseket. Így válik láthatóvá, kinek a hangja hiányzik a sátorból. Egy óra ilyenkor sok idő, és a sátor előtt várakozó katonák nem értik, miért nem indulnak még.</t>
         </is>
       </c>
       <c r="H8" s="18" t="n">
@@ -5716,7 +5716,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="76" customHeight="1">
+    <row r="9" ht="90" customHeight="1">
       <c r="A9" s="15" t="n"/>
       <c r="B9" s="16" t="n"/>
       <c r="C9" s="17" t="n"/>
@@ -5727,7 +5727,7 @@
       </c>
       <c r="E9" s="17" t="inlineStr">
         <is>
-          <t>Vargára hallgatsz: ő a szakember, ő ismeri a gátakat. A városi töltésre összpontosítotok, a gazdák csalódottan mennek haza.</t>
+          <t>Vargára hallgatsz: ő a szakember, ő ismeri a gátakat. A városi töltésre összpontosítotok, a gazdák pedig csalódottan mennek haza.</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">
@@ -5737,7 +5737,7 @@
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet csoportos döntési modelljei között szerepel a szakértői döntés: a csoport azt hagyja dönteni, aki a kérdésben a legjáratosabb. A gátakról Varga tud a legtöbbet, ez erős érv. A modell hátránya, hogy nincs benne párbeszéd, és a döntés súlya — negyven család megélhetése — egy mérnöki szempontra szűkül.</t>
+          <t>A jegyzet csoportos döntési modelljei között szerepel a szakértői döntés: a csoport azt hagyja dönteni, aki az adott kérdésben a legjáratosabb. A gátakról valóban Varga tud a legtöbbet, és ez erős érv. A modell hátránya, hogy nincs benne párbeszéd, és egy ekkora súlyú döntés — negyven család megélhetése — egyetlen mérnöki szempontra szűkül.</t>
         </is>
       </c>
       <c r="H9" s="18" t="n">
@@ -5770,12 +5770,12 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Két előrejelzés</t>
+          <t>Két eltérő előrejelzés</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>A dandárparancsnokság minden reggel hatkor egyetlen számot kér: mekkora lesz a tetőzés. Csakhogy két előrejelzés van. Az egyik hét méter húsz centit mond, a másik hét méter kilencvenet — a városi gát hét méter hatvanig biztos. A rádión várják a jelentésedet.</t>
+          <t>A dandárparancsnokság minden reggel hatkor egyetlen számot kér: mekkora lesz a tetőzés. Csakhogy két előrejelzés van. Az egyik hét méter húsz centit mond, a másik hét méter kilencvenet, a városi gát pedig hét méter hatvanig biztosan tart. A rádió túloldalán a jelentésedet várják.</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -5785,7 +5785,7 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Mindkét számot jelented, és mindkettőhöz leírod, mit csinálsz, ha az jön be. A parancsnokság bosszús, mert egyetlen számot kért.</t>
+          <t>Mindkét számot jelented, és mindkettőhöz leírod, mit teszel, ha az következik be. A parancsnokság bosszús, mert egyetlen számot kért.</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Snowden és Boone összetett helyzetnek nevezik, amikor az ok-okozati viszonyok felderíthetők, de nem azonnal láthatók, és több helyes válasz is létezhet — ilyenkor szakértői mérlegelésre van szükség. Két előrejelzés éppen ilyen helyzet, és te nem tettél úgy, mintha csak egy lenne. A pontos kép bosszantja azokat, akik egyszerű választ vártak.</t>
+          <t>Snowden és Boone összetett helyzetnek nevezi, amikor az ok-okozati összefüggések feltárhatók, de nem azonnal láthatók, és több helyes válasz is létezhet — ilyenkor szakértői mérlegelésre van szükség. A két előrejelzés éppen ilyen helyzetet teremt, és te nem tettél úgy, mintha csak egy volna. A pontos kép viszont bosszantja azokat, akik egyszerű választ vártak.</t>
         </is>
       </c>
       <c r="H10" s="12" t="n">
@@ -5833,7 +5833,7 @@
       </c>
       <c r="E11" s="17" t="inlineStr">
         <is>
-          <t>Megkéred a törzsfőnököt, hogy jöjjön ki, és nézze meg a helyszínt a saját szemével, mielőtt a számokról döntenek. Ezzel a parancsnokságon nem szerzel barátokat.</t>
+          <t>Megkéred a törzsfőnököt, hogy jöjjön ki, és a saját szemével nézze meg a helyszínt, mielőtt döntenek a számokról. Ezzel nem szerzel jó pontot a parancsnokságon.</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg kapcsolattartó szerepében a vezető olyan emberekkel tart kapcsolatot, akik maguk is információs központok. Ha a törzsfőnök látja a töltést, a számok mögött a valóságot is érti. A kérés viszont a szolgálati utat kerüli meg, és van, aki ezt okoskodásnak fogja venni.</t>
+          <t>Mintzberg kapcsolattartó szerepében a vezető olyan emberekkel tart kapcsolatot, akik maguk is információs csomópontok. Ha a törzsfőnök látja a töltést, a számok mögött a valóságot is érti. A kérés viszont megkerüli a szolgálati utat, és lesz, aki ezt okoskodásnak tartja majd.</t>
         </is>
       </c>
       <c r="H11" s="18" t="n">
@@ -5891,7 +5891,7 @@
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>A szelektív hárítás az, amikor a kellemetlen, félelmetes információt nem engedjük be, mert zavarja a képet, amelyet fenn akarunk tartani. Az indokaid valódiak: a pánik tényleg veszélyes. De ha a magasabb szám jön be, a parancsnokság olyan helyzetre készült, amely nem létezik.</t>
+          <t>Szelektív hárításról akkor beszélünk, amikor a kellemetlen, ijesztő információt nem engedjük be, mert zavarja azt a képet, amelyet fenn akarunk tartani. Az indokaid valósak: a pánik tényleg veszélyes. Ha viszont a magasabb szám jön be, a parancsnokság egy olyan helyzetre készült fel, amely nem létezik.</t>
         </is>
       </c>
       <c r="H12" s="18" t="n">
@@ -5929,7 +5929,7 @@
       </c>
       <c r="E13" s="17" t="inlineStr">
         <is>
-          <t>A magasabb számot jelented, hogy biztosan kapj még két gépet és egy századot. Ha nem jön be, legfeljebb túlbiztosítottátok.</t>
+          <t>A magasabb számot jelented, hogy biztosan kapj még két gépet és egy századot. Ha mégsem jön be, legfeljebb túlbiztosítottátok magatokat.</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
@@ -5939,7 +5939,7 @@
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg tárgyaló szerepében a vezető erőforrásokat szerez a szervezetének egyezkedés útján. A magasabb számmal jó eséllyel megkapod az erősítést, amelyre szükséged lehet. Ha viszont kiderül, hogy a jelentésedet a céljaidhoz igazítottad, legközelebb a pontos számaidnak sem fognak hinni.</t>
+          <t>Mintzberg tárgyaló szerepében a vezető egyezkedéssel szerez erőforrásokat a szervezetének. A magasabb számmal jó eséllyel megkapod az erősítést, amelyre szükséged lehet. Ha viszont kiderül, hogy a jelentésedet a saját céljaidhoz igazítottad, legközelebb a pontos számaidnak sem fognak hinni.</t>
         </is>
       </c>
       <c r="H13" s="18" t="n">
@@ -5966,18 +5966,18 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="76" customHeight="1">
+    <row r="14" ht="90" customHeight="1">
       <c r="A14" s="9" t="n">
         <v>4</v>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Egy gép, két szakasz</t>
+          <t>Egy markoló, két gátszakasz</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>A harmadik napon két helyen is gyengül a töltés: a városi gátnál egy rövidebb, a tanyák felett egy hosszabb szakaszon. Egyetlen nagy teljesítményű markolótok van. A két szakaszparancsnok egyszerre hív a rádión, és mindkettő a gépet kéri.</t>
+          <t>A harmadik napon két helyen is gyengülni kezd a töltés: a városi gátnál egy rövidebb, a tanyák felett egy hosszabb szakaszon. Egyetlen nagy teljesítményű markolótok van. A két szakaszparancsnok egyszerre hív a rádión, és mindketten a gépet kérik.</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
@@ -5987,7 +5987,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>A városé az elsőbbség: emberek előbb, mint a termés. Ezt szabályként mondod ki, és mindkét parancsnok tudja, mihez tartsa magát.</t>
+          <t>A város élvez elsőbbséget: előbb az emberek, aztán a termés. Ezt szabályként mondod ki, így mindkét parancsnok tudja, mihez tartsa magát.</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
@@ -5997,7 +5997,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Simon szerint a jól strukturált döntésnél világos, mi a probléma, a rosszul strukturáltnál viszont nem. Egy egyszerű szabállyal jól strukturálttá tetted a helyzetet, és ez gyors, kiszámítható parancsokat ad. A szabály azonban elrejti, hogy a tanyáknál is emberek élnek, és ha ott szakad át a gát, a „csak termés” nem lesz igaz.</t>
+          <t>Simon szerint a jól strukturált döntésnél világos, mi a probléma, a rosszul strukturáltnál viszont nem. Egy egyszerű szabállyal jól strukturálttá tetted a helyzetet, és ez gyors, kiszámítható parancsokat tesz lehetővé. A szabály azonban elfedi, hogy a tanyákon is emberek élnek, és ha ott szakad át a gát, ott sem „csak a termés” lesz veszélyben.</t>
         </is>
       </c>
       <c r="H14" s="12" t="n">
@@ -6045,7 +6045,7 @@
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>Az inkrementalizmus nagy döntések helyett kis, fokozatos lépéseket jelent, amelyek közben a helyzet alakulásához lehet igazodni. A váltás egyik szakaszt sem hagyja magára, és a legkönnyebben megtehető lépés. Csakhogy az átállás idő, és könnyen lehet, hogy estére mindkét szakasz félkész marad.</t>
+          <t>Az inkrementalizmus azt jelenti, hogy nagy döntések helyett kis, fokozatos lépésekben haladunk, és közben igazodunk a helyzet alakulásához. A váltott munka egyik szakaszt sem hagyja magára, és ez a legkönnyebben megtehető lépés. Csakhogy az átállás is időbe telik, és könnyen lehet, hogy estére mindkét szakasz félkész marad.</t>
         </is>
       </c>
       <c r="H15" s="18" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="E16" s="17" t="inlineStr">
         <is>
-          <t>Felírjátok, melyik szakasz mögött hány ház, hány ember és mennyi termés van, és mennyi idő a javítás. Először megnézitek, van-e olyan lehetőség, amelyik mindenben rosszabb egy másiknál. Ez húsz perc a rádió mellett.</t>
+          <t>Végiggondoljátok, melyik szakasz mögött hány ház, hány ember és mennyi termés van, és mennyi idő a javítás. Először megnézitek, van-e olyan lehetőség, amelyik minden szempontból rosszabb egy másiknál. Ez húsz perc a rádió mellett.</t>
         </is>
       </c>
       <c r="F16" s="17" t="inlineStr">
@@ -6093,7 +6093,7 @@
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
-          <t>A dominancia elve szerint ha egy lehetőség semmiben nem jobb egy másiknál, és legalább egy szempontból rosszabb, azt nyugodtan elvethetjük, mielőtt nehezebb mérlegelésbe kezdenénk. Ha az egyik szakasz minden szempontból kevésbé sürgős, a döntés magától megszületik. Ha nem, legalább tudod, min múlik — de húsz percig mindkét szakasz vár.</t>
+          <t>A dominancia elve szerint ha egy lehetőség semmiben sem jobb egy másiknál, és legalább egy szempontból rosszabb, nyugodtan elvethetjük, mielőtt nehezebb mérlegelésbe kezdenénk. Ha az egyik szakasz minden szempontból kevésbé sürgős, a döntés magától megszületik. Ha nem, legalább tudod, min múlik a választás — de húsz percig mindkét szakasz vár.</t>
         </is>
       </c>
       <c r="H16" s="18" t="n">
@@ -6131,7 +6131,7 @@
       </c>
       <c r="E17" s="17" t="inlineStr">
         <is>
-          <t>Bérelsz egy második gépet egy helyi vállalkozótól a saját keretedből, amihez nincs engedélyed. Utólag kell majd elszámolnod vele.</t>
+          <t>Bérelsz egy második gépet egy helyi vállalkozótól a saját keretedből, bár erre nincs engedélyed. Utólag kell majd elszámolnod vele.</t>
         </is>
       </c>
       <c r="F17" s="17" t="inlineStr">
@@ -6141,7 +6141,7 @@
       </c>
       <c r="G17" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg vállalkozó szerepében a vezető maga kezdeményez változást, és felkutatja a lehetőségeket. A második géppel kilépsz a „vagy-vagy” helyzetből, és mindkét szakasz megkapja, amit kér. Ennek ára a szabálysértés: ha a dandár nem fogadja el az elszámolást, a döntés a te nevedhez kötődik.</t>
+          <t>Mintzberg vállalkozó szerepében a vezető maga kezdeményez változást, és maga kutatja fel a lehetőségeket. A második géppel kilépsz a „vagy-vagy” helyzetből, és mindkét szakasz megkapja, amit kér. Ennek ára a szabályszegés: ha a dandár nem fogadja el az elszámolást, a döntés a te nevedhez fűződik.</t>
         </is>
       </c>
       <c r="H17" s="18" t="n">
@@ -6174,12 +6174,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Műszaki hiba</t>
+          <t>A hamis naplóbejegyzés</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Az ötödik éjjel megsérül egy katona: húsz órája volt talpon, és elesett a gép mellett. Takács százados a naplóba ennyit írt: baleset, műszaki hiba. A dandár reggel hatkor olvassa a jelentést. Ha kiderül a kimerültség, vizsgálat indul, és pihenőt kell elrendelni — pont most, amikor minden kéz kell.</t>
+          <t>Az ötödik éjjel megsérül egy katona: húsz órája volt talpon, és megbotlott a markoló mellett. Takács százados ennyit írt a naplóba: baleset, műszaki hiba. A dandár reggel hatkor olvassa a jelentést. Ha kiderül, hogy a baleset oka a kimerültség volt, vizsgálat indul, és pihenőt kell elrendelni — éppen most, amikor minden kézre szükség van.</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
@@ -6189,7 +6189,7 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Kijavíttatod a naplót: kimerültség miatt történt. És azonnal kötelező pihenőt vezetsz be, még ha kevesebben is maradnak a gátnál.</t>
+          <t>Kijavíttatod a naplót: a baleset kimerültség miatt történt. Emellett azonnal kötelező pihenőt vezetsz be, még ha így kevesebben maradnak is a gátnál.</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -6199,7 +6199,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>A napfény teszt egyetlen kérdés: jól érezném magam, ha ez a döntés minden részletével együtt nyilvánosságra kerülne? Egy elhallgatott kimerültségi baleset ezt nem állná ki, főleg ha később valaki súlyosabban sérül. A pontos napló és a pihenő a helyes lépés, de a gátnál most kevesebb kéz marad.</t>
+          <t>A napfény teszt egyetlen kérdés: jól érezném-e magam, ha ez a döntés minden részletével együtt nyilvánosságra kerülne? Egy kimerültség miatti baleset eltussolása ezt nem állná ki, különösen, ha később valaki súlyosabban megsérül. A pontos napló és a pihenő a helyes lépés, de a gátnál most kevesebb kéz marad.</t>
         </is>
       </c>
       <c r="H18" s="12" t="n">
@@ -6226,7 +6226,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="76" customHeight="1">
+    <row r="19" ht="90" customHeight="1">
       <c r="A19" s="15" t="n"/>
       <c r="B19" s="16" t="n"/>
       <c r="C19" s="17" t="n"/>
@@ -6237,7 +6237,7 @@
       </c>
       <c r="E19" s="17" t="inlineStr">
         <is>
-          <t>A bejegyzés marad: most minden ember kell, egy vizsgálat most megbénítaná a védekezést. A kérdést a víz levonulása után rendezed.</t>
+          <t>A bejegyzés marad: most minden emberre szükség van, és egy vizsgálat megbénítaná a védekezést. A kérdést a víz levonulása után rendezed.</t>
         </is>
       </c>
       <c r="F19" s="17" t="inlineStr">
@@ -6247,7 +6247,7 @@
       </c>
       <c r="G19" s="17" t="inlineStr">
         <is>
-          <t>A diszkontálás az a hajlamunk, hogy ami közel van, azt felértékeljük, ami távolabb, azt leértékeljük. A következő két nap védekezése most mindennél fontosabbnak látszik, a hamis bejegyzés következményei pedig távolinak. Csakhogy a kimerültség attól még ott van, és a következő baleset már nem biztos, hogy ilyen könnyű lesz.</t>
+          <t>A diszkontálás az a hajlamunk, hogy ami közel van, azt túlértékeljük, ami távolabb esik, azt pedig alábecsüljük. A következő két nap védekezése most mindennél fontosabbnak tűnik, a hamis bejegyzés következményei pedig távolinak. A kimerültség azonban ettől még megmarad, és nem biztos, hogy a következő baleset is ilyen enyhe lesz.</t>
         </is>
       </c>
       <c r="H19" s="18" t="n">
@@ -6274,7 +6274,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="76" customHeight="1">
+    <row r="20" ht="90" customHeight="1">
       <c r="A20" s="15" t="n"/>
       <c r="B20" s="16" t="n"/>
       <c r="C20" s="17" t="n"/>
@@ -6285,7 +6285,7 @@
       </c>
       <c r="E20" s="17" t="inlineStr">
         <is>
-          <t>Megkérdezed a századparancsnokokat és néhány katonát, mit gondolnak, és velük együtt döntitek el, hogyan legyen a pihenő és mi kerüljön a jelentésbe.</t>
+          <t>Megkérdezed a századparancsnokokat és néhány katonát, mit gondolnak, és velük együtt döntitek el, hogyan legyen megszervezve a pihenő, és mi kerüljön a jelentésbe.</t>
         </is>
       </c>
       <c r="F20" s="17" t="inlineStr">
@@ -6295,7 +6295,7 @@
       </c>
       <c r="G20" s="17" t="inlineStr">
         <is>
-          <t>A részvételi létra azt mutatja, mennyire valódi a bevonás: puszta tájékoztatás, meghallgatás vagy tényleges beleszólás a döntésbe. Az állomány most beleszólhat abba, ami a saját biztonságáról szól, és ezt komolyan fogják venni. A jelentés tartalma viszont a te parancsnoki felelősséged, és ezt nem lehet szavazásra bocsátani.</t>
+          <t>A részvételi létra azt mutatja meg, mennyire valódi a bevonás: puszta tájékoztatás, meghallgatás vagy tényleges beleszólás a döntésbe. Az állomány most beleszólhat abba, ami a saját biztonságát érinti, és ezt komolyan is fogják venni. A jelentés tartalma viszont a te parancsnoki felelősséged, és azt nem lehet szavazásra bocsátani.</t>
         </is>
       </c>
       <c r="H20" s="18" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="E21" s="17" t="inlineStr">
         <is>
-          <t>A bejegyzés marad, de csendben bevezetsz egy pihenőrendet. A katonák kipihentebbek lesznek, és senkinek nem esik bántódása.</t>
+          <t>A bejegyzés marad, de csendben bevezetsz egy pihenőrendet. A katonák kipihentebbek lesznek, és senkinek sem esik bántódása.</t>
         </is>
       </c>
       <c r="F21" s="17" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="G21" s="17" t="inlineStr">
         <is>
-          <t>A gátló racionalizálások olyan érvek, amelyekkel egy kétes lépést magunk előtt elfogadhatóvá teszünk. A „senkinek sem árt” szerint ha nincs közvetlen károsult, a döntés rendben van. A pihenőrend valóban véd, de a hamis napló megmarad, és ha kiderül, a jó szándék már nem fog számítani.</t>
+          <t>A gátló racionalizálások olyan érvek, amelyekkel egy kétes lépést a saját szemünkben elfogadhatóvá teszünk. A „senkinek sem árt” logikája szerint ha nincs közvetlen károsult, a döntés rendben van. A pihenőrend valóban védi az embereket, de a hamis bejegyzés megmarad, és ha kiderül, a jó szándék már nem fog számítani.</t>
         </is>
       </c>
       <c r="H21" s="18" t="n">
@@ -6376,12 +6376,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>A legelők</t>
+          <t>Legelők elárasztása kártérítésért</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>A hatodik napon a felvízi falu két vezetője ül le veled a rádióasztalhoz. Ha átengeditek a vizet a legelőikre, a városi gát megmenekülhet. Beleegyeznek — de csak akkor, ha írásban garantálod a kártérítést. Ezt nem a te hatásköröd megígérni, a minisztériumi döntés pedig napokig tarthat.</t>
+          <t>A hatodik napon a folyó felső szakaszán fekvő falu két vezetője ül le veled a rádióasztalhoz. Ha átengeditek a vizet a legelőikre, a városi gát megmenekülhet. Beleegyeznek — de csak akkor, ha írásban garantálod a kártérítést. Ennek megígérése nem a te hatásköröd, a minisztérium döntése pedig napokig is eltarthat.</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
@@ -6391,7 +6391,7 @@
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>Megígéred a kártérítést, és aláírod a papírt. A víz még ma éjjel a legelőkre mehet, a garanciát majd utólag elintézed.</t>
+          <t>Megígéred a kártérítést, és aláírod a papírt. A víz még ma éjjel a legelőkre mehet, a garanciát pedig majd utólag elintézed.</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
@@ -6401,7 +6401,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>James March hamisan pozitív hibának nevezi, amikor a döntéshozó olyan kontrollban hisz, amely a valóságban nincs meg. A kártérítés nem a te kezedben van, mégis úgy írtad alá, mintha az lenne. A város ma éjjel biztonságosabb, de ha a minisztérium nem fizet, a falu soha többé nem fog hinni egy katonai aláírásnak.</t>
+          <t>James March hamisan pozitív hibának nevezi, amikor a döntéshozó olyan kontrollban hisz, amely a valóságban nincs a kezében. A kártérítésről nem te döntesz, mégis úgy írtad alá, mintha rajtad múlna. A város ma éjjel nagyobb biztonságban van, de ha a minisztérium nem fizet, a falu soha többé nem fog hinni egy katonai aláírásnak.</t>
         </is>
       </c>
       <c r="H22" s="12" t="n">
@@ -6439,7 +6439,7 @@
       </c>
       <c r="E23" s="17" t="inlineStr">
         <is>
-          <t>Életvédelmi helyzetre hivatkozva elrendeled a víz átengedését a falu beleegyezése nélkül. A törvény erre lehetőséget ad, de a falu bizalma elveszik.</t>
+          <t>Életveszélyre hivatkozva a falu beleegyezése nélkül elrendeled a víz átengedését. A törvény erre lehetőséget ad, de a falu bizalmát elveszíted.</t>
         </is>
       </c>
       <c r="F23" s="17" t="inlineStr">
@@ -6449,7 +6449,7 @@
       </c>
       <c r="G23" s="17" t="inlineStr">
         <is>
-          <t>Az autokratikus döntésnél a vezető egyedül dönt, az érintettek közreműködése nélkül. A jegyzet szerint ez válsághelyzetben, időhiányban indokolt lehet, és most valóban emberéletek a tét. A falu viszont nem partner, hanem elszenvedője lett a döntésnek, és ezt a következő árvíznél is fel fogja idézni.</t>
+          <t>Az autokratikus döntésnél a vezető egyedül dönt, az érintettek bevonása nélkül. A jegyzet szerint ez válsághelyzetben, időhiány esetén indokolt lehet, és most valóban emberéletek forognak kockán. A falu viszont nem partnere, hanem elszenvedője lett a döntésnek, és ezt a következő árvíznél is fel fogja hozni.</t>
         </is>
       </c>
       <c r="H23" s="18" t="n">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="E24" s="17" t="inlineStr">
         <is>
-          <t>Nem teszel semmit, amíg a minisztériumtól meg nem jön az írásos felhatalmazás. A szabályok szerint jársz el, de közben a víz tovább emelkedik.</t>
+          <t>Nem teszel semmit, amíg meg nem érkezik a minisztérium írásos felhatalmazása. A szabályok szerint jársz el, de közben a víz tovább emelkedik.</t>
         </is>
       </c>
       <c r="F24" s="17" t="inlineStr">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="G24" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet a döntéshozói magatartások között írja le a passzív alkalmazkodást: korlátozott hit abban, hogy befolyásolni tudjuk a dolgokat, és a meglévő szabályok, struktúrák elfogadása. Szabályosan jársz el, ezt senki nem vetheti a szemedre. Közben viszont éppen a legjobb lehetőség csúszik ki a kezedből.</t>
+          <t>A jegyzet a döntéshozói magatartások között írja le a passzív alkalmazkodást: a vezető kevéssé hisz abban, hogy befolyásolni tudja az eseményeket, és elfogadja a meglévő szabályokat és struktúrákat. Szabályosan jársz el, ezt senki sem vetheti a szemedre. Közben viszont éppen a legjobb lehetőség csúszik ki a kezedből.</t>
         </is>
       </c>
       <c r="H24" s="18" t="n">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="E25" s="17" t="inlineStr">
         <is>
-          <t>Őszintén elmondod, mit tudsz megígérni és mit nem, és a kérésüket azonnal továbbítod a minisztériumnak. Lehet, hogy így nemet mondanak, és elveszítitek a legjobb esélyt.</t>
+          <t>Őszintén elmondod, mit tudsz megígérni és mit nem, és a kérésüket azonnal továbbítod a minisztériumnak. Lehet, hogy így nemet mondanak, és elszalasztjátok a legjobb esélyt.</t>
         </is>
       </c>
       <c r="F25" s="17" t="inlineStr">
@@ -6545,7 +6545,7 @@
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg szóvivő szerepében a vezető a kívülállóknak pontosan elmondja, mit tesz a szervezete és mit nem. Az őszinte „ezt nem ígérhetem meg” hitelesebb minden garanciánál, és a falu is tudja, mire számíthat. Ennek ára, hogy a megállapodás elcsúszhat, és a víz közben nem vár.</t>
+          <t>Mintzberg szóvivő szerepében a vezető pontosan elmondja a kívülállóknak, mit vállal a szervezete és mit nem. Egy őszinte „ezt nem ígérhetem meg” hitelesebb minden garanciánál, és a falu is tudja, mire számíthat. Ennek ára, hogy a megállapodás késhet, a víz pedig közben nem vár.</t>
         </is>
       </c>
       <c r="H25" s="18" t="n">
@@ -6578,12 +6578,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Hét kilencven</t>
+          <t>Három terv, kevés idő</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>A hetedik este új előrejelzés érkezik: hajnalra hét méter kilencven. A tervasztalon három lehetőség fekszik: egész éjjel magasítjátok a városi gátat homokzsákkal; kitelepítitek a város alsó részét; vagy mindent a felvízi tározásra tesztek. A tisztjeid mind mást javasolnak, és kevés az idő.</t>
+          <t>A hetedik este új előrejelzés érkezik: hajnalra hét méter kilencven centi lesz a vízszint. Három lehetőség közül választhatsz: egész éjjel homokzsákokkal magasítjátok a városi gátat, kitelepítitek a város alsó részét, vagy mindent a folyón feljebb lévő tározóra tesztek fel. A tisztjeid mind mást javasolnak, és kevés az idő.</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
@@ -6593,7 +6593,7 @@
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>A kitelepítést rendeled el: ha az emberek biztonságban vannak, a házakat még meg lehet védeni vagy újjáépíteni. A pánik és a kifosztástól való félelem viszont a te számládra megy.</t>
+          <t>Elrendeled a kitelepítést: ha az emberek biztonságban vannak, a házakat még meg lehet védeni vagy újjá lehet építeni. A pánik és a fosztogatástól való félelem viszont a te lelkeden szárad.</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
@@ -6603,7 +6603,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>A PrOACT-modell második lépése a célok tisztázása: mit akarunk mindenképp elérni, és mit akarunk elkerülni? Te kimondtad, hogy az emberélet minden más cél előtt áll, és ehhez igazítottad a döntést. Ez világos rangsor, de ára is van: elhagyott házak, dühös lakók, és egy éjszaka, amelyet a város sokáig nem felejt.</t>
+          <t>A PrOACT-modell második lépése a célok tisztázása: mit akarunk mindenképp elérni, és mit akarunk elkerülni? Te kimondtad, hogy az emberélet minden más célt megelőz, és ehhez igazítottad a döntést. Ez világos rangsor, de ára is van: elhagyott házak, dühös lakók, és egy éjszaka, amelyet a város sokáig nem felejt el.</t>
         </is>
       </c>
       <c r="H26" s="12" t="n">
@@ -6641,7 +6641,7 @@
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>Mindhárom tervet egyszerre indítod el, szétosztva az embereket. Így egyik lehetőségről sem mondasz le, de mindegyikre kevesebb erő jut.</t>
+          <t>Mindhárom tervet egyszerre indítod el, és szétosztod köztük az embereket. Így egyik lehetőségről sem mondasz le, de mindegyikre kevesebb erő jut.</t>
         </is>
       </c>
       <c r="F27" s="17" t="inlineStr">
@@ -6651,7 +6651,7 @@
       </c>
       <c r="G27" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg erőforrás-elosztó szerepében a vezető dönti el, hová kerül az ember és az eszköz, és ezzel alapvetően meghatározza, mire képesek az egységek. Mindhárom tervre adni valamennyit biztonságosnak tűnik, és senki nem érzi mellőzöttnek magát. Könnyen lehet viszont, hogy hajnalra egyik terv sem kap annyi erőt, amennyi a sikerhez kellett volna.</t>
+          <t>Mintzberg erőforrás-elosztó szerepében a vezető dönti el, hová kerülnek az emberek és az eszközök, és ezzel alapvetően meghatározza, mire képesek az egységek. Biztonságosnak tűnik mindhárom tervnek adni valamennyit, és így senki sem érzi magát mellőzöttnek. Könnyen lehet viszont, hogy hajnalra egyik terv sem kap annyi erőt, amennyi a sikerhez kellett volna.</t>
         </is>
       </c>
       <c r="H27" s="18" t="n">
@@ -6689,7 +6689,7 @@
       </c>
       <c r="E28" s="17" t="inlineStr">
         <is>
-          <t>Megkéred a tiszteket, hogy tíz percig mindenki egyedül írja le, mit tart jónak és miért, és csak utána beszélitek meg. Tíz perc éjjel sok idő.</t>
+          <t>Megkéred a tiszteket, hogy tíz percig mindenki egyedül gondolja át, mit tart jónak és miért, és csak utána beszélitek meg. Éjjel tíz perc sok idő.</t>
         </is>
       </c>
       <c r="F28" s="17" t="inlineStr">
@@ -6699,7 +6699,7 @@
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
-          <t>A névleges csoport módszerben a tagok először egymástól függetlenül gondolkodnak, és csak utána osztják meg az ötleteiket. Így nem a rangidős vagy a leghangosabb érvei köré rendeződik a vita, és a csendesebb tisztek is megszólalnak. Az ára a tíz perc, ami ebben a helyzetben valódi áldozat.</t>
+          <t>A névleges csoport módszerben a tagok először egymástól függetlenül gondolkodnak, és csak utána osztják meg az ötleteiket. Így a vita nem a rangidős vagy a leghangosabb ember érvei köré rendeződik, és a csendesebb tisztek is szóhoz jutnak. Az ára a tíz perc, ami ebben a helyzetben valódi áldozat.</t>
         </is>
       </c>
       <c r="H28" s="18" t="n">
@@ -6737,7 +6737,7 @@
       </c>
       <c r="E29" s="17" t="inlineStr">
         <is>
-          <t>A tapasztalatodra hagyatkozol: a homokzsákos magasítás eddig minden árvíznél bevált, és ezt ismerik a katonák is.</t>
+          <t>A tapasztalatodra hagyatkozol: a homokzsákos magasítás eddig minden árvíznél bevált, és a katonák is ismerik.</t>
         </is>
       </c>
       <c r="F29" s="17" t="inlineStr">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="G29" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet szerint a sémák a korábbi tapasztalatokból épülő gondolkodási minták, amelyek segítenek gyorsan dönteni, de makaccsá is válhatnak. A homokzsák bevált séma, és a katonák ismerik a feladatot. Csakhogy ez az árhullám magasabb minden eddiginél, és a séma éppen azt nem mutatja meg, miben más ez az éjszaka.</t>
+          <t>A jegyzet szerint a sémák korábbi tapasztalatokra épülő gondolkodási minták, amelyek segítenek gyorsan dönteni, de merevvé is tehetnek. A homokzsák bevált séma, és a katonák ismerik a feladatot. Csakhogy ez az árhullám minden eddiginél magasabb, és a séma éppen azt nem mutatja meg, miben más ez az éjszaka.</t>
         </is>
       </c>
       <c r="H29" s="18" t="n">
@@ -6780,12 +6780,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Bakos bácsi</t>
+          <t>A gátőr figyelmeztetése</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Hajnali kettőkor Bakos Feri bácsi, a nyugdíjas gátőr kivezet a régi töltéshez. A töltés tövében tiszta víz szivárog. Varga mérnök szerint ez csak esővíz, nincs vele teendő. Az öreg ragaszkodik hozzá: 1970-ben pontosan így kezdődött a szakadás. Emberből és homokzsákból is kevés van.</t>
+          <t>Hajnali kettőkor Bakos Feri bácsi, a nyugdíjas gátőr kivezet a régi töltéshez. A töltés tövében tiszta víz szivárog. Varga mérnök szerint ez csak esővíz, nincs vele teendő. Az öreg azonban kitart: 1970-ben pontosan így kezdődött a gátszakadás. Emberből és homokzsákból is kevés van.</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
@@ -6795,7 +6795,7 @@
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>Vargára hallgatsz: ő a mérnök, az öreg csak aggódik. Megköszönöd a figyelmességét, és hazaküldöd.</t>
+          <t>Vargára hallgatsz: ő a mérnök, az öreg csak aggódik. Megköszönöd Bakos bácsinak a figyelmességét, és hazaküldöd.</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
@@ -6805,7 +6805,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Az ezredes-hatás az a hajlamunk, hogy a magasabb beosztású vagy nagyobb tekintélyű ember szavát hitelesebbnek tartsuk. Varga szakember, és gyakran igaza van — de a beosztása önmagában nem bizonyíték. Az erőid a városi gátnál maradnak, egy lehetséges figyelmeztetés viszont válasz nélkül maradt.</t>
+          <t>Az ezredes-hatás az a hajlamunk, hogy a magasabb beosztású vagy nagyobb tekintélyű ember szavát hitelesebbnek tartjuk. Varga szakember, és gyakran igaza van — de a beosztása önmagában nem bizonyíték. Az erőid a városi gátnál maradnak, egy lehetséges figyelmeztetésre viszont senki sem reagált.</t>
         </is>
       </c>
       <c r="H30" s="12" t="n">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="G31" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet szerint ha hiányzik egy információ, hajlamosak vagyunk feltevésekkel vagy pletykákkal kitölteni a hézagot. Te nem Vargának vagy Bakos bácsinak adtál igazat, hanem ténnyel pótoltad a hiányzó darabot: ha a szivárgó víz zavaros, a töltés belseje mosódik. Ez a legjobb információ, amit szerezhetsz, de fél órát tart, és addig te tartod a kockázatot.</t>
+          <t>A jegyzet szerint ha hiányzik egy információ, hajlamosak vagyunk feltevésekkel vagy szóbeszéddel kitölteni a hézagot. Te nem Vargának vagy Bakos bácsinak adtál igazat, hanem ténnyel pótoltad a hiányzó darabot: ha a szivárgó víz zavaros, akkor a töltés belseje mosódik ki. Ez a legjobb információ, amelyhez hozzájuthatsz, de fél órába telik, és addig a kockázat a tiéd.</t>
         </is>
       </c>
       <c r="H31" s="18" t="n">
@@ -6880,7 +6880,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="76" customHeight="1">
+    <row r="32" ht="90" customHeight="1">
       <c r="A32" s="15" t="n"/>
       <c r="B32" s="16" t="n"/>
       <c r="C32" s="17" t="n"/>
@@ -6891,7 +6891,7 @@
       </c>
       <c r="E32" s="17" t="inlineStr">
         <is>
-          <t>Bakos bácsira hallgatsz: odaküldesz egy szakaszt homokzsákkal, Varga ellenkezése ellenére. A városi gát ezzel gyengébb lesz.</t>
+          <t>Bakos bácsira hallgatsz: Varga ellenkezése ellenére odaküldesz egy szakaszt homokzsákokkal. Ezzel a városi gát védelme gyengül.</t>
         </is>
       </c>
       <c r="F32" s="17" t="inlineStr">
@@ -6901,7 +6901,7 @@
       </c>
       <c r="G32" s="17" t="inlineStr">
         <is>
-          <t>A sztereotipizálás az, amikor valakit a csoport alapján ítélünk meg, ahová tartozik — például egy nyugdíjast „aggódó öregnek”. Te nem estél ebbe a csapdába: Bakos bácsi ötven év tapasztalatát adatnak tekintetted. Ennek ára, hogy a mérnököt felülbírálod, és egy erősen fenyegetett gátról vonsz el embert.</t>
+          <t>Sztereotipizálásról akkor beszélünk, amikor valakit aszerint ítélünk meg, milyen csoporthoz tartozik — például egy nyugdíjast „aggódó öregnek” tekintünk. Te nem estél ebbe a csapdába: Bakos bácsi ötvenévnyi tapasztalatát valódi adatként kezelted. Ennek ára, hogy felülbírálod a mérnököt, és egy erősen veszélyeztetett gáttól vonsz el embereket.</t>
         </is>
       </c>
       <c r="H32" s="18" t="n">
@@ -6949,7 +6949,7 @@
       </c>
       <c r="G33" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet háromféle vezetői stratégiát különít el: a problémakeresőt, a problémamegoldót és a problémakerülőt. A két ember közös helyszíni bejárása jó ötlet, és talán meg is egyeznek. A döntés súlya viszont nem az övék: ha nem jutnak dűlőre, a vitájuk alatt a töltés nem vár.</t>
+          <t>A jegyzet háromféle vezetői stratégiát különít el: a problémakeresőt, a problémamegoldót és a problémakerülőt. Jó ötlet, hogy ketten együtt nézzék meg a helyszínt, és talán meg is egyeznek. A döntés súlya azonban nem az ő vállukat nyomja: ha nem jutnak dűlőre, a töltés nem vár, amíg vitatkoznak.</t>
         </is>
       </c>
       <c r="H33" s="18" t="n">
@@ -6982,12 +6982,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Húsz ház</t>
+          <t>A gátszakadás után</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Hajnali fél ötkor a régi töltés egy szakaszon átszakad. A víz a mezőkre és a város szélére ömlik: senki nem hal meg, de húsz ház víz alá kerül. Reggel az állomány sorakozik. Kimerültek, megrendültek, és már terjed a hír, hogy a parancsnokság hibázott. A városi gát még tart, a munka folytatódik.</t>
+          <t>Hajnali fél ötkor a régi töltés egy szakaszon átszakad. A víz a mezőkre és a város szélére ömlik: senki sem hal meg, de húsz ház víz alá kerül. Reggel az állomány sorakozik. Kimerültek és megrendültek, és már terjed a hír, hogy a parancsnokság hibázott. A városi gát még tart, a munka folytatódik.</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
@@ -6997,7 +6997,7 @@
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>A víz erejét hangsúlyozod: ezt senki nem akadályozhatta volna meg, mindenki a legjobbat adta. Ez megnyugtatja a katonákat.</t>
+          <t>A víz erejét hangsúlyozod: ezt senki sem akadályozhatta volna meg, mindenki a legjobbját adta. Ez megnyugtatja a katonákat.</t>
         </is>
       </c>
       <c r="F34" s="11" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Az énmegerősítő attribúció az a hajlamunk, hogy a kudarcot a körülményeknek, a sikert saját magunknak tulajdonítsuk. A megnyugtatás most valóban kell, és a víz ereje valóban óriási volt. De ha a döntések szerepe ki sem mondódik, az állomány a pletykából fogja megtudni, amit tőled nem hallott.</t>
+          <t>Az énmegerősítő attribúció az a hajlamunk, hogy a kudarcot a körülményeknek, a sikert pedig saját magunknak tulajdonítjuk. A megnyugtatásra most valóban szükség van, és a víz ereje tényleg óriási volt. Ha azonban a döntések szerepéről egy szó sem esik, az állomány a pletykákból tudja meg azt, amit tőled nem hallott.</t>
         </is>
       </c>
       <c r="H34" s="12" t="n">
@@ -7055,7 +7055,7 @@
       </c>
       <c r="G35" s="17" t="inlineStr">
         <is>
-          <t>Snowden és Boone szerint kaotikus helyzetben nincs idő elemezni: először cselekedni kell, hogy a helyzet stabilizálódjon, és csak utána érdemes keresni az okokat. A városi gát tartása valóban ilyen feladat. Csakhogy a hallgatás is üzenet, és a kimerült emberek fejében a pletyka tölti ki az űrt.</t>
+          <t>Snowden és Boone szerint kaotikus helyzetben nincs idő elemzésre: először cselekedni kell, hogy a helyzet stabilizálódjon, és csak utána érdemes az okokat keresni. A városi gát megtartása valóban ilyen feladat. Csakhogy a hallgatás is üzenet, és a kimerült emberek fejében a pletyka tölti ki az űrt.</t>
         </is>
       </c>
       <c r="H35" s="18" t="n">
@@ -7082,7 +7082,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="62" customHeight="1">
+    <row r="36" ht="76" customHeight="1">
       <c r="A36" s="15" t="n"/>
       <c r="B36" s="16" t="n"/>
       <c r="C36" s="17" t="n"/>
@@ -7093,7 +7093,7 @@
       </c>
       <c r="E36" s="17" t="inlineStr">
         <is>
-          <t>Előbb a századparancsnokoktól kérdezed meg, mit hallanak az emberektől, és csak utána szólsz az állományhoz. Addig mindenki vár.</t>
+          <t>Előbb a századparancsnokoktól kérdezed meg, mit hallanak az emberektől, és csak ezután szólsz az állományhoz. Addig mindenki vár.</t>
         </is>
       </c>
       <c r="F36" s="17" t="inlineStr">
@@ -7103,7 +7103,7 @@
       </c>
       <c r="G36" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg információgyűjtő szerepében a vezető a belső információáramlás központja. Ha tudod, mit beszélnek az emberek, pontosan azokra a kérdésekre válaszolhatsz, amelyek bennük vannak. Az ára a várakozás egy olyan reggelen, amikor minden perc a gáté.</t>
+          <t>Mintzberg információgyűjtő szerepében a vezető a szervezeten belüli információáramlás központja. Ha tudod, mit beszélnek az emberek, pontosan azokra a kérdésekre válaszolhatsz, amelyek őket foglalkoztatják. Az ára a várakozás egy olyan reggelen, amikor minden perc a gáté.</t>
         </is>
       </c>
       <c r="H36" s="18" t="n">
@@ -7141,7 +7141,7 @@
       </c>
       <c r="E37" s="17" t="inlineStr">
         <is>
-          <t>Kiállsz eléjük, és elmondod, mi történt, mi volt benne a te döntésed, és mi a következő huszonnégy óra feladata.</t>
+          <t>Kiállsz eléjük, és elmondod, mi történt, mi volt ebben a te döntésed, és mi a feladat a következő huszonnégy órában.</t>
         </is>
       </c>
       <c r="F37" s="17" t="inlineStr">
@@ -7151,7 +7151,7 @@
       </c>
       <c r="G37" s="17" t="inlineStr">
         <is>
-          <t>Mintzberg vezető szerepe a vezető és a beosztottai közötti viszonyról szól, és ez hatja át az egész vezetői munkát. Ha a nehéz pillanatban is kiállsz, és vállalod a saját részedet, az állomány tudja, hogy a parancsnokának szavára lehet építeni. A beismerés viszont a dandárnál ellened is fordítható, és egy darabig megingathatja a parancsnoki lánc önbizalmát.</t>
+          <t>Mintzberg vezető szerepe a vezető és a beosztottai közötti viszonyról szól, és ez az egész vezetői munkát áthatja. Ha a nehéz pillanatban is kiállsz, és vállalod a saját részedet, az állomány tudja, hogy számíthat a parancsnoka szavára. A beismerést viszont a dandárnál ellened is fordíthatják, és egy időre megingathatja a parancsnoki lánc önbizalmát.</t>
         </is>
       </c>
       <c r="H37" s="18" t="n">
@@ -7184,12 +7184,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>A vizsgálat</t>
+          <t>Jelentés a vizsgálóbizottságnak</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>A tizenkettedik napon a víz levonul. A dandár vizsgálóbizottsága a te értékelésedet kéri: mi történt, és ki miért felel. A naplóbejegyzés, a régi töltés és a gép körüli döntések mind benne lesznek. Amit leírsz, emberek pályáját döntheti el — a sajátodat is.</t>
+          <t>A tizenkettedik napon levonul a víz. A dandár vizsgálóbizottsága a te értékelésedet kéri: mi történt, és ki miért felel. A naplóbejegyzés, a régi töltés és a markoló körüli döntések mind szóba kerülnek. Amit leírsz, emberek pályáját döntheti el — a tiédet is.</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
@@ -7209,7 +7209,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Az alapvető attribúciós hiba az a hajlamunk, hogy mások hibáját a jellemükkel, a sajátunkat a körülményekkel magyarázzuk. Takács hibája valódi, de ő is ugyanabban a kimerítő helyzetben dolgozott, mint mindenki. Ha csak őt nevezed meg, a jelentés igaz lesz — és mégis egyoldalú.</t>
+          <t>Az alapvető attribúciós hiba az a hajlamunk, hogy mások hibáját a jellemükkel, a sajátunkat pedig a körülményekkel magyarázzuk. Takács hibája valódi, de ő is ugyanolyan kimerítő körülmények között dolgozott, mint mindenki más. Ha csak őt nevezed meg, a jelentés igaz lesz, mégis egyoldalú.</t>
         </is>
       </c>
       <c r="H38" s="12" t="n">
@@ -7247,7 +7247,7 @@
       </c>
       <c r="E39" s="17" t="inlineStr">
         <is>
-          <t>Mindent leírsz, a saját hibáidat is, névvel és döntéssel együtt. A jelentés így hiteles, de a karriered is benne van.</t>
+          <t>Mindent leírsz, a saját hibáidat is, névvel és döntéssel együtt. A jelentés így hiteles, de a karriered is a tét.</t>
         </is>
       </c>
       <c r="F39" s="17" t="inlineStr">
@@ -7257,7 +7257,7 @@
       </c>
       <c r="G39" s="17" t="inlineStr">
         <is>
-          <t>A következtetési létra azt mutatja be, milyen gyorsan jutunk a tényekből feltevésekhez és döntésekhez; a reflektív gondolkodás ezen a létrán való tudatos lemászás. Ha a saját feltevéseidet is végigveszed, a jelentés tanulsággá válik, nem vádirattá. Ennek ára a saját pályád kockázata, és az, hogy a feletteseid ezt nem mindig fogják értékelni.</t>
+          <t>A következtetési létra azt mutatja be, milyen gyorsan jutunk el a tényektől a feltevésekig és a döntésekig; a reflektív gondolkodás azt jelenti, hogy tudatosan visszamászunk ezen a létrán. Ha a saját feltevéseidet is végiggondolod, a jelentésből tanulság lesz, nem vádirat. Ennek ára, hogy a saját pályádat kockáztatod, és a feletteseid ezt nem mindig fogják értékelni.</t>
         </is>
       </c>
       <c r="H39" s="18" t="n">
@@ -7295,7 +7295,7 @@
       </c>
       <c r="E40" s="17" t="inlineStr">
         <is>
-          <t>A jelentést a tisztjeiddel közösen írjátok meg, és a polgármestert, a gazdákat és Bakos bácsit is meghallgatjátok. Így teljesebb lesz a kép, de a felelősség is szétterül.</t>
+          <t>A jelentést a tisztjeiddel közösen írjátok meg, és a polgármestert, a gazdákat és Bakos bácsit is meghallgatjátok. Így teljesebb lesz a kép, de a felelősség is szétoszlik.</t>
         </is>
       </c>
       <c r="F40" s="17" t="inlineStr">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="G40" s="17" t="inlineStr">
         <is>
-          <t>A jegyzet szerint a csoportos döntések során megoszlik a felelősség, a valóban bevont résztvevők pedig elkötelezettebbé válnak. A közös jelentés több nézőpontot hoz, és a helyiek is úgy érzik, számított, amit átéltek. Az ára, hogy a te parancsnoki felelősséged elmosódhat a sok hang között.</t>
+          <t>A jegyzet szerint csoportos döntésnél megoszlik a felelősség, a valóban bevont résztvevők pedig jobban elköteleződnek. A közös jelentés több nézőpontot mutat be, és a helyiek is úgy érzik, hogy számított, amit átéltek. Az ára, hogy a te parancsnoki felelősséged elmosódhat a sok hang között.</t>
         </is>
       </c>
       <c r="H40" s="18" t="n">
@@ -7343,7 +7343,7 @@
       </c>
       <c r="E41" s="17" t="inlineStr">
         <is>
-          <t>A rendszer hibáit írod le — kevés gép, pontatlan előrejelzés, ellentmondó utasítások —, személyeket nem nevezel meg. Ez igaz is, és senki pályája nem törik meg.</t>
+          <t>A rendszer hibáit írod le — kevés gép, pontatlan előrejelzés, egymásnak ellentmondó utasítások —, személyeket nem nevezel meg. Ez igaz is, és így senkinek sem törik meg a pályája.</t>
         </is>
       </c>
       <c r="F41" s="17" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="G41" s="17" t="inlineStr">
         <is>
-          <t>James March hamisan negatív hibának nevezi, amikor a döntéshozó azt feltételezi, hogy a dolgok menetére nem volt befolyása, pedig lehetett volna. A rendszerhibák valósak, és jó, hogy leírod őket. Ha viszont csak ezeket látod, a jelentésből kimarad, hol lehetett volna másként dönteni, és a következő árvíznél ugyanazok a döntések születnek.</t>
+          <t>James March hamisan negatív hibának nevezi, amikor a döntéshozó azt feltételezi, hogy nem volt befolyása az események alakulására, pedig lehetett volna. A rendszerhibák valósak, és jó, hogy leírod őket. Ha viszont csak ezeket látod, a jelentésből kimarad, hol lehetett volna másként dönteni, és a következő árvíznél ugyanezek a döntések születnek majd.</t>
         </is>
       </c>
       <c r="H41" s="18" t="n">

</xml_diff>